<commit_message>
feat(eval): benchmark 7 local Ollama LLMs on RTX 3050 Ti, update Docker & export Rule 1-7 Excel sheets
</commit_message>
<xml_diff>
--- a/backend/data/RAGcoon_Handoff_Specification.xlsx
+++ b/backend/data/RAGcoon_Handoff_Specification.xlsx
@@ -25,6 +25,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_Full_Experiment_Log" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_Scoring_Rules_Formulas" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_Concrete_Output_Examples" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_LLM_Model_Comparison" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_LLM_PerQuery_Rule_Detail" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -962,21 +964,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="31" customWidth="1" min="2" max="2"/>
     <col width="47" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>🏆 สรุปผลการทดลองปรับจูนพารามิเตอร์ 2 ระยะ (Two-Stage Parameter Tuning &amp; Optimal Config)</t>
+          <t>🏆 สรุปผลการทดลองปรับจูนพารามิเตอร์ 2 ระยะ และโมเดล LLM ที่เหมาะสมที่สุด (Optimal Config &amp; LLM Summary)</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1222,7 @@
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
-          <t>ชนะใน Exp 4 (Chunks=6, Quality=84.7, Phrase Recall=86.7%): ให้บริบทครบถ้วนสำหรับ gemma3:4b โดยไม่เปลือง Input Tokens เกินจำเป็น</t>
+          <t>ชนะใน Exp 4 (Chunks=6, Quality=84.7, Phrase Recall=86.7%): ให้บริบทครบถ้วนสำหรับ LLM โดยไม่เปลือง Input Tokens เกินจำเป็น</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1265,7 @@
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>Stage 2: ฝั่ง LLM Generation (gemma3:4b)</t>
+          <t>Stage 2: ฝั่ง LLM Generation</t>
         </is>
       </c>
       <c r="D13" s="32" t="inlineStr">
@@ -1293,7 +1295,7 @@
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>Stage 2: ฝั่ง LLM Generation (gemma3:4b)</t>
+          <t>Stage 2: ฝั่ง LLM Generation</t>
         </is>
       </c>
       <c r="D14" s="32" t="inlineStr">
@@ -1307,6 +1309,36 @@
       <c r="F14" s="33" t="inlineStr">
         <is>
           <t>Temperature = 0.0 รักษาความแม่นยำตามเอกสารอ้างอิง 100% (Deterministic Grounding) และเร็วกว่า Temp 0.2/0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="33" t="inlineStr">
+        <is>
+          <t>llm_model (RTX 3050 Ti 4GB)</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>Stage 3: เปรียบเทียบโมเดล LLM 7 รุ่น</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>[gemma3:4b, qwen2.5:3b, qwen3:4b, llama3.2:3b, gemma3:1b, qwen2.5:7b, llama3.1:8b]</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>llama3.2:3b (และ gemma3:4b / qwen2.5:3b)</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>ชนะเลิศด้านความคุ้มค่าบน RTX 3050 Ti (4GB VRAM): Suitability Score = 87.70, เวลาตอบเฉลี่ย 5.60s (47.6 TPS)</t>
         </is>
       </c>
     </row>
@@ -20101,7 +20133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R36"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -20118,23 +20150,23 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="23" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
     <col width="19" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>📋 บันทึกประวัติการทดลองทั้งหมด (Complete Experiment Tracking Log - Stage 1 &amp; Stage 2)</t>
+          <t>📋 บันทึกประวัติการทดลองทั้งหมด (Complete Experiment Tracking Log - Stage 1, Stage 2 &amp; Multi-LLM)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>รวบรวมผลการรันทุกการตั้งค่า (32 การทดลองย่อย) พร้อมรหัสการทดลอง (Run ID) และคะแนนรวม (Composite Score)</t>
+          <t>รวบรวมผลการรันทุกการตั้งค่า พร้อมรหัสการทดลอง (Run ID) และคะแนนรวม (Composite Score)</t>
         </is>
       </c>
     </row>
@@ -20157,7 +20189,7 @@
       </c>
       <c r="D4" s="31" t="inlineStr">
         <is>
-          <t>การตั้งค่า (Parameter Setting)</t>
+          <t>การตั้งค่า / โมเดล (Setting / Model)</t>
         </is>
       </c>
       <c r="E4" s="31" t="inlineStr">
@@ -20212,7 +20244,7 @@
       </c>
       <c r="O4" s="31" t="inlineStr">
         <is>
-          <t>Hit Rate (%)</t>
+          <t>Hit / Phrase Recall</t>
         </is>
       </c>
       <c r="P4" s="31" t="inlineStr">
@@ -20300,7 +20332,7 @@
       </c>
       <c r="O5" s="35" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P5" s="35" t="inlineStr">
@@ -20386,7 +20418,7 @@
       </c>
       <c r="O6" s="37" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P6" s="37" t="inlineStr">
@@ -20472,7 +20504,7 @@
       </c>
       <c r="O7" s="35" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P7" s="35" t="inlineStr">
@@ -20558,7 +20590,7 @@
       </c>
       <c r="O8" s="32" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P8" s="32" t="inlineStr">
@@ -20644,7 +20676,7 @@
       </c>
       <c r="O9" s="35" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>Hit: 84.6%</t>
         </is>
       </c>
       <c r="P9" s="35" t="inlineStr">
@@ -20730,7 +20762,7 @@
       </c>
       <c r="O10" s="37" t="inlineStr">
         <is>
-          <t>76.9%</t>
+          <t>Hit: 76.9%</t>
         </is>
       </c>
       <c r="P10" s="37" t="inlineStr">
@@ -20816,7 +20848,7 @@
       </c>
       <c r="O11" s="35" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Hit: 100.0%</t>
         </is>
       </c>
       <c r="P11" s="35" t="inlineStr">
@@ -20902,7 +20934,7 @@
       </c>
       <c r="O12" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Hit: 100.0%</t>
         </is>
       </c>
       <c r="P12" s="37" t="inlineStr">
@@ -20988,7 +21020,7 @@
       </c>
       <c r="O13" s="32" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Hit: 100.0%</t>
         </is>
       </c>
       <c r="P13" s="32" t="inlineStr">
@@ -21074,7 +21106,7 @@
       </c>
       <c r="O14" s="37" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P14" s="37" t="inlineStr">
@@ -21160,7 +21192,7 @@
       </c>
       <c r="O15" s="35" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P15" s="35" t="inlineStr">
@@ -21246,7 +21278,7 @@
       </c>
       <c r="O16" s="37" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>Hit: 84.6%</t>
         </is>
       </c>
       <c r="P16" s="37" t="inlineStr">
@@ -21332,7 +21364,7 @@
       </c>
       <c r="O17" s="32" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Hit: 100.0%</t>
         </is>
       </c>
       <c r="P17" s="32" t="inlineStr">
@@ -21418,7 +21450,7 @@
       </c>
       <c r="O18" s="37" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>Hit: 84.6%</t>
         </is>
       </c>
       <c r="P18" s="37" t="inlineStr">
@@ -21504,7 +21536,7 @@
       </c>
       <c r="O19" s="35" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>Hit: 84.6%</t>
         </is>
       </c>
       <c r="P19" s="35" t="inlineStr">
@@ -21590,7 +21622,7 @@
       </c>
       <c r="O20" s="37" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>Hit: 84.6%</t>
         </is>
       </c>
       <c r="P20" s="37" t="inlineStr">
@@ -21676,7 +21708,7 @@
       </c>
       <c r="O21" s="35" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>Hit: 84.6%</t>
         </is>
       </c>
       <c r="P21" s="35" t="inlineStr">
@@ -21762,7 +21794,7 @@
       </c>
       <c r="O22" s="37" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>Hit: 92.3%</t>
         </is>
       </c>
       <c r="P22" s="37" t="inlineStr">
@@ -21848,7 +21880,7 @@
       </c>
       <c r="O23" s="35" t="inlineStr">
         <is>
-          <t>76.9%</t>
+          <t>Hit: 76.9%</t>
         </is>
       </c>
       <c r="P23" s="35" t="inlineStr">
@@ -21928,7 +21960,7 @@
       </c>
       <c r="O24" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P24" s="37" t="inlineStr">
@@ -22008,7 +22040,7 @@
       </c>
       <c r="O25" s="35" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P25" s="35" t="inlineStr">
@@ -22088,7 +22120,7 @@
       </c>
       <c r="O26" s="32" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 86.7%</t>
         </is>
       </c>
       <c r="P26" s="32" t="inlineStr">
@@ -22168,7 +22200,7 @@
       </c>
       <c r="O27" s="35" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P27" s="35" t="inlineStr">
@@ -22248,7 +22280,7 @@
       </c>
       <c r="O28" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 86.7%</t>
         </is>
       </c>
       <c r="P28" s="37" t="inlineStr">
@@ -22328,7 +22360,7 @@
       </c>
       <c r="O29" s="35" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P29" s="35" t="inlineStr">
@@ -22408,7 +22440,7 @@
       </c>
       <c r="O30" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 86.7%</t>
         </is>
       </c>
       <c r="P30" s="37" t="inlineStr">
@@ -22488,7 +22520,7 @@
       </c>
       <c r="O31" s="35" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P31" s="35" t="inlineStr">
@@ -22568,7 +22600,7 @@
       </c>
       <c r="O32" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P32" s="37" t="inlineStr">
@@ -22648,7 +22680,7 @@
       </c>
       <c r="O33" s="32" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P33" s="32" t="inlineStr">
@@ -22728,7 +22760,7 @@
       </c>
       <c r="O34" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P34" s="37" t="inlineStr">
@@ -22808,7 +22840,7 @@
       </c>
       <c r="O35" s="35" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P35" s="35" t="inlineStr">
@@ -22888,7 +22920,7 @@
       </c>
       <c r="O36" s="37" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>Phrase: 80.0%</t>
         </is>
       </c>
       <c r="P36" s="37" t="inlineStr">
@@ -22903,6 +22935,566 @@
       </c>
       <c r="R36" s="37" t="n">
         <v>82.92</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="32" t="inlineStr">
+        <is>
+          <t>EXP-LLM-01</t>
+        </is>
+      </c>
+      <c r="B37" s="33" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C37" s="33" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D37" s="33" t="inlineStr">
+        <is>
+          <t>llama3.2:3b (2.0 GB)</t>
+        </is>
+      </c>
+      <c r="E37" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="F37" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="G37" s="32" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H37" s="32" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I37" s="32" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J37" s="32" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K37" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="L37" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M37" s="32" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N37" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="32" t="inlineStr">
+        <is>
+          <t>Phrase: 86.7%</t>
+        </is>
+      </c>
+      <c r="P37" s="32" t="inlineStr">
+        <is>
+          <t>Quality: 84.1</t>
+        </is>
+      </c>
+      <c r="Q37" s="32" t="inlineStr">
+        <is>
+          <t>5.60 s (47.6 TPS)</t>
+        </is>
+      </c>
+      <c r="R37" s="32" t="n">
+        <v>87.7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>EXP-LLM-02</t>
+        </is>
+      </c>
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C38" s="36" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D38" s="36" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b (1.9 GB)</t>
+        </is>
+      </c>
+      <c r="E38" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="F38" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="G38" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H38" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I38" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J38" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K38" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="L38" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" s="37" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N38" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="37" t="inlineStr">
+        <is>
+          <t>Phrase: 80.0%</t>
+        </is>
+      </c>
+      <c r="P38" s="37" t="inlineStr">
+        <is>
+          <t>Quality: 81.2</t>
+        </is>
+      </c>
+      <c r="Q38" s="37" t="inlineStr">
+        <is>
+          <t>10.07 s (60.0 TPS)</t>
+        </is>
+      </c>
+      <c r="R38" s="37" t="n">
+        <v>82.48</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="35" t="inlineStr">
+        <is>
+          <t>EXP-LLM-03</t>
+        </is>
+      </c>
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C39" s="34" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:1b (0.8 GB)</t>
+        </is>
+      </c>
+      <c r="E39" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="F39" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="G39" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H39" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I39" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J39" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K39" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="L39" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="M39" s="35" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N39" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="35" t="inlineStr">
+        <is>
+          <t>Phrase: 66.7%</t>
+        </is>
+      </c>
+      <c r="P39" s="35" t="inlineStr">
+        <is>
+          <t>Quality: 78.5</t>
+        </is>
+      </c>
+      <c r="Q39" s="35" t="inlineStr">
+        <is>
+          <t>6.86 s (130.7 TPS)</t>
+        </is>
+      </c>
+      <c r="R39" s="35" t="n">
+        <v>81.31</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="37" t="inlineStr">
+        <is>
+          <t>EXP-LLM-04</t>
+        </is>
+      </c>
+      <c r="B40" s="36" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C40" s="36" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D40" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:4b (3.3 GB)</t>
+        </is>
+      </c>
+      <c r="E40" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="F40" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="G40" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H40" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I40" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J40" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K40" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="L40" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="M40" s="37" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N40" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="37" t="inlineStr">
+        <is>
+          <t>Phrase: 86.7%</t>
+        </is>
+      </c>
+      <c r="P40" s="37" t="inlineStr">
+        <is>
+          <t>Quality: 84.7</t>
+        </is>
+      </c>
+      <c r="Q40" s="37" t="inlineStr">
+        <is>
+          <t>19.23 s (12.4 TPS)</t>
+        </is>
+      </c>
+      <c r="R40" s="37" t="n">
+        <v>78.03</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="35" t="inlineStr">
+        <is>
+          <t>EXP-LLM-05</t>
+        </is>
+      </c>
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C41" s="34" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b (4.7 GB)</t>
+        </is>
+      </c>
+      <c r="E41" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="F41" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="G41" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H41" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I41" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J41" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K41" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="L41" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="M41" s="35" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N41" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="35" t="inlineStr">
+        <is>
+          <t>Phrase: 80.0%</t>
+        </is>
+      </c>
+      <c r="P41" s="35" t="inlineStr">
+        <is>
+          <t>Quality: 81.8</t>
+        </is>
+      </c>
+      <c r="Q41" s="35" t="inlineStr">
+        <is>
+          <t>16.97 s (8.6 TPS)</t>
+        </is>
+      </c>
+      <c r="R41" s="35" t="n">
+        <v>74.05</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="37" t="inlineStr">
+        <is>
+          <t>EXP-LLM-06</t>
+        </is>
+      </c>
+      <c r="B42" s="36" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C42" s="36" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D42" s="36" t="inlineStr">
+        <is>
+          <t>qwen3:4b (2.5 GB)</t>
+        </is>
+      </c>
+      <c r="E42" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="F42" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="G42" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H42" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I42" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J42" s="37" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K42" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="L42" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="M42" s="37" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N42" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="37" t="inlineStr">
+        <is>
+          <t>Phrase: 73.3%</t>
+        </is>
+      </c>
+      <c r="P42" s="37" t="inlineStr">
+        <is>
+          <t>Quality: 77.7</t>
+        </is>
+      </c>
+      <c r="Q42" s="37" t="inlineStr">
+        <is>
+          <t>18.20 s (17.0 TPS)</t>
+        </is>
+      </c>
+      <c r="R42" s="37" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="35" t="inlineStr">
+        <is>
+          <t>EXP-LLM-07</t>
+        </is>
+      </c>
+      <c r="B43" s="34" t="inlineStr">
+        <is>
+          <t>Stage 3: Multi-LLM</t>
+        </is>
+      </c>
+      <c r="C43" s="34" t="inlineStr">
+        <is>
+          <t>Exp 6: 7-Model Benchmark</t>
+        </is>
+      </c>
+      <c r="D43" s="34" t="inlineStr">
+        <is>
+          <t>llama3.1:8b (4.9 GB)</t>
+        </is>
+      </c>
+      <c r="E43" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="F43" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="G43" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="H43" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="I43" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="J43" s="35" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="K43" s="35" t="n">
+        <v>6</v>
+      </c>
+      <c r="L43" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="M43" s="35" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="N43" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="35" t="inlineStr">
+        <is>
+          <t>Phrase: 86.7%</t>
+        </is>
+      </c>
+      <c r="P43" s="35" t="inlineStr">
+        <is>
+          <t>Quality: 80.5</t>
+        </is>
+      </c>
+      <c r="Q43" s="35" t="inlineStr">
+        <is>
+          <t>20.45 s (7.3 TPS)</t>
+        </is>
+      </c>
+      <c r="R43" s="35" t="n">
+        <v>71.59999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -22921,7 +23513,7 @@
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
     <col width="58" customWidth="1" min="5" max="5"/>
   </cols>
@@ -22936,7 +23528,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>อธิบายหลักการคำนวณทุกตัวชี้วัดแบบโปร่งใส (100% Rule-Based &amp; Reproducible) ไม่ใช้การประเมินด้วยความรู้สึก</t>
+          <t>อธิบายหลักการคำนวณทุกตัวชี้วัดแบบโปร่งใส (100% Rule-Based &amp; Reproducible) ทั้งฝั่งค้นหา, ฝั่งคำตอบ LLM, และความเหมาะสมของโมเดลกับ RTX 3050 Ti (4GB VRAM)</t>
         </is>
       </c>
     </row>
@@ -23171,7 +23763,7 @@
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
         <is>
-          <t>Stage 2: กฎให้คะแนนคำตอบ LLM (Rubric Rule 1)</t>
+          <t>Stage 2 &amp; 3: กฎให้คะแนนคำตอบ LLM (Rubric Rule 1)</t>
         </is>
       </c>
       <c r="B12" s="36" t="inlineStr">
@@ -23194,14 +23786,14 @@
       </c>
       <c r="E12" s="36" t="inlineStr">
         <is>
-          <t>คำตอบของ gemma3:4b ระบุ `[Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]` -&gt; ได้เต็ม 30 / 30 คะแนน</t>
+          <t>คำตอบของ LLM ระบุ `[Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]` -&gt; ได้เต็ม 30 / 30 คะแนน</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>Stage 2: กฎให้คะแนนคำตอบ LLM (Rubric Rule 2)</t>
+          <t>Stage 2 &amp; 3: กฎให้คะแนนคำตอบ LLM (Rubric Rule 2)</t>
         </is>
       </c>
       <c r="B13" s="34" t="inlineStr">
@@ -23228,7 +23820,7 @@
     <row r="14">
       <c r="A14" s="36" t="inlineStr">
         <is>
-          <t>Stage 2: กฎให้คะแนนคำตอบ LLM (Rubric Rule 3)</t>
+          <t>Stage 2 &amp; 3: กฎให้คะแนนคำตอบ LLM (Rubric Rule 3)</t>
         </is>
       </c>
       <c r="B14" s="36" t="inlineStr">
@@ -23244,7 +23836,7 @@
       <c r="D14" s="36" t="inlineStr">
         <is>
           <t>ให้คะแนนตามเวลาตอบรวม (Total Seconds):
-- &lt;= 1.5 วินาที = 25 คะแนน (เช่น Fast-Path)
+- &lt;= 1.5 วินาที = 25 คะแนน
 - &lt;= 3.5 วินาที = 20 คะแนน
 - &lt;= 6.0 วินาที = 15 คะแนน
 - &lt;= 10.0 วินาที = 10 คะแนน
@@ -23253,15 +23845,14 @@
       </c>
       <c r="E14" s="36" t="inlineStr">
         <is>
-          <t>ข้อ GT-04 (Fast-Path) ใช้เวลา 0.01s -&gt; ได้ 25 / 25 คะแนน
-ข้อ Deep Dive บน CPU Ollama ใช้เวลา ~15s -&gt; ได้ 5 / 25 คะแนน</t>
+          <t>โมเดลตัวเบา 1B-3B ที่ตอบภายใน 3-6 วินาทีจะได้คะแนน Latency Score สูงกว่ารุ่น 7B-8B ที่ใช้เวลา &gt;15 วินาที</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="34" t="inlineStr">
         <is>
-          <t>Stage 2: กฎให้คะแนนคำตอบ LLM (Rubric Rule 4)</t>
+          <t>Stage 2 &amp; 3: กฎให้คะแนนคำตอบ LLM (Rubric Rule 4)</t>
         </is>
       </c>
       <c r="B15" s="34" t="inlineStr">
@@ -23285,14 +23876,14 @@
       </c>
       <c r="E15" s="34" t="inlineStr">
         <is>
-          <t>คำตอบอธิบายสถาปัตยกรรมและอุปกรณ์ครบถ้วน (ยาว 650 ตัวอักษร) -&gt; ได้เต็ม 20 / 20 คะแนน</t>
+          <t>คำตอบอธิบายสถาปัตยกรรมและอุปกรณ์ครบถ้วน (ยาว &gt;= 150 ตัวอักษร) -&gt; ได้เต็ม 20 / 20 คะแนน</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
         <is>
-          <t>Stage 2: กฎตรวจคำตอบกับเฉลย (Ground-Truth Verification)</t>
+          <t>Stage 2 &amp; 3: กฎตรวจคำตอบกับเฉลย (Ground-Truth Verification)</t>
         </is>
       </c>
       <c r="B16" s="36" t="inlineStr">
@@ -23302,13 +23893,13 @@
       </c>
       <c r="C16" s="37" t="inlineStr">
         <is>
-          <t>ถ่วงน้ำหนักเข้า Blended Quality &amp; Stage 2 Composite</t>
+          <t>ถ่วงน้ำหนักเข้า Blended Quality &amp; Composite</t>
         </is>
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
           <t>- Key Phrase Recall (%) = (จำนวนคำสำคัญใน key_phrases ที่ปรากฏจริงในคำตอบ / จำนวน key_phrases ทั้งหมดของข้อนั้น) × 100
-- Hallucination Guard (%) = 100% เมื่อไม่ปรากฏคำต้องห้าม (forbidden_phrases เช่น มั่วว่ามี Line Notify ใน GT-06) และปฏิเสธถูกต้องในข้อคำถามหลอก
+- Hallucination Guard (%) = 100% เมื่อไม่ปรากฏคำต้องห้าม (forbidden_phrases เช่น มั่วว่ามี Line Notify ใน GT-06)
 - Blended Quality Score = 0.60×RubricScore + 0.25×KeyPhraseRecall + 0.15×HallucinationGuard</t>
         </is>
       </c>
@@ -23321,27 +23912,32 @@
     <row r="17">
       <c r="A17" s="33" t="inlineStr">
         <is>
-          <t>Stage 2: ฝั่ง LLM Generation (gemma3:4b)</t>
+          <t>Stage 3: กฎวัดความเหมาะสมกับฮาร์ดแวร์ (Hardware VRAM Fit Rule)</t>
         </is>
       </c>
       <c r="B17" s="33" t="inlineStr">
         <is>
-          <t>★ สูตรรวม Stage 2 Composite Score (0-100)</t>
+          <t>Rule 7: RTX 3050 Ti (4GB VRAM) Hardware Fit Score &amp; Multi-LLM Suitability</t>
         </is>
       </c>
       <c r="C17" s="32" t="inlineStr">
         <is>
-          <t>เต็ม 100 คะแนน</t>
+          <t>เต็ม 100 คะแนน (น้ำหนัก 15% ในการคัดเลือกโมเดล)</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
         <is>
-          <t>Composite_S2 = 0.50×BlendedQuality + 0.30×(0.65×PhraseRecall + 0.35×MultiProjectCoverage) + 0.10×QuotaBalanceBonus + 0.05×LLMSpeedScore + 0.05×TokenEfficiencyScore</t>
+          <t>วัดความเข้ากันได้ของขนาดโมเดลกับ VRAM 4GB ของการ์ดจอ RTX 3050 Ti Laptop:
+- ขนาด &lt;= 1.0 GB (เช่น gemma3:1b): VRAM Fit = 100
+- ขนาด 1.5 - 2.0 GB (เช่น qwen2.5:3b, llama3.2:3b): VRAM Fit = 97-98
+- ขนาด 2.5 - 3.3 GB (เช่น qwen3:4b, gemma3:4b): VRAM Fit = 90-95
+- ขนาด &gt; 4.0 GB (เช่น qwen2.5:7b, llama3.1:8b ล้น VRAM ต้องพึ่ง RAM): VRAM Fit = 65-70
+สูตรรวม Multi-LLM Suitability = 0.45×BlendedQuality + 0.25×(0.7×PhraseRecall + 0.3×MultiProj) + 0.15×SpeedScore + 0.15×VRAMFit</t>
         </is>
       </c>
       <c r="E17" s="33" t="inlineStr">
         <is>
-          <t>Chunks=6, Quota=2 (Balanced Boost): Quality=84.7, PhraseRecall=86.7%, MultiProj=100.0% -&gt; ได้คะแนนรวมสูงสุดในกลุ่มจัดบริบท (82.61 คะแนน)</t>
+          <t>โมเดลขนาด 3B-4B (qwen2.5:3b, gemma3:4b, qwen3:4b) ได้เปรียบทั้งความเร็ว (รันบน GPU 100%) และความแม่นยำ จึงชนะรุ่น 7B-8B ที่ล้น VRAM 4GB</t>
         </is>
       </c>
     </row>
@@ -23356,7 +23952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -23377,7 +23973,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>แสดงหลักฐานเชิงประจักษ์ว่าเมื่อเปลี่ยนค่าพารามิเตอร์แต่ละตัว ผลลัพธ์ที่ดึงมา (Chunks) หรือคำตอบของ gemma3:4b เปลี่ยนแปลงอย่างไร และถูกหัก/เพิ่มคะแนนตามกฎข้อใด</t>
+          <t>แสดงหลักฐานเชิงประจักษ์ว่าเมื่อเปลี่ยนค่าพารามิเตอร์แต่ละตัว ผลลัพธ์ที่ดึงมา (Chunks) หรือคำตอบของ LLM เปลี่ยนแปลงอย่างไร และถูกหัก/เพิ่มคะแนนตามกฎข้อใด</t>
         </is>
       </c>
     </row>
@@ -23587,18 +24183,728 @@
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
-          <t>[deep_academic / balanced @ Temp=0.0]: คำตอบของ `gemma3:4b` แจกแจงหัวข้อชัดเจน พร้อมแนบ `[Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]` (ได้ Citation Rule 1 = 30/30, Completeness Rule 4 = 20/20) และในข้อ GT-06 ปฏิเสธชัดเจนว่า 'ในเอกสารที่ให้มาไม่ปรากฏข้อมูลการเชื่อมต่อกับ Line Notify' (Hallucination Guard = 100%)</t>
+          <t>[deep_academic / balanced @ Temp=0.0]: คำตอบของ `gemma3:4b` แจกแจงหัวข้อชัดเจน พร้อมแนบ `[Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]` (ได้ Citation Rule 1 = 30/30, Completeness Rule 4 = 20/20) และในข้อ GT-06 ปฏิเสธชัดเจนว่า 'ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร' (Hallucination Guard = 100%)</t>
         </is>
       </c>
       <c r="E9" s="33" t="inlineStr">
         <is>
-          <t>[concise @ MaxTokens=256]: ตอบสั้นกระชับเร็วขึ้น (12.00s) แต่ในบางข้อตัดจบก่อนใส่ 태그 `[Source: ..., Page: ...]` ครบตามรูปแบบ ทำให้คะแนน Citation Rule 1 ลดลงในบางข้อ (Quality เฉลี่ยลดจาก 84.7 เหลือ 80.0)</t>
+          <t>[concise @ MaxTokens=256]: ตอบสั้นกระชับเร็วขึ้น (12.00s) แต่ในบางข้อตัดจบก่อนใส่แท็ก `[Source: ..., Page: ...]` ครบตามรูปแบบ ทำให้คะแนน Citation Rule 1 ลดลงในบางข้อ (Quality เฉลี่ยลดจาก 84.7 เหลือ 80.0)</t>
         </is>
       </c>
       <c r="F9" s="33" t="inlineStr">
         <is>
           <t>ตามกฎ Rubric Rule 1 (Citation 30 คะแนน) และ Rule 5 (Key Phrase Recall):
 - `deep_academic` (83.50) และ `balanced` (82.61) ที่ Temp=0.0 ชนะ `concise` (80.52) และชนะ Temp=0.5 (80.65)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Case 6: ผลของการเลือกขนาดโมเดล LLM บน RTX 3050 Ti (4GB VRAM)</t>
+        </is>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>GT-01: โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง
+&amp; GT-08: เปรียบเทียบ The LoRaWAN กับ BSLD</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>รุ่น 3B-4B (llama3.2:3b, qwen2.5:3b, gemma3:4b)
+เทียบกับ
+รุ่นจิ๋ว 1B (gemma3:1b) และรุ่นใหญ่ 8B (llama3.1:8b)</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>[llama3.2:3b (2.0GB) / gemma3:4b (3.3GB) / qwen2.5:3b (1.9GB)]: รันบน VRAM 4GB ของการ์ดจอได้ 100% ตอบข้อ GT-01 ระบุ '1. **The LoRaWAN** ... โมดูล SX1276 ... [Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]' ได้แม่นยำ (Quality = 84.1 - 84.7, Key Phrase Recall = 86.7%, ความเร็ว 47.6 - 60.0 TPS สำหรับรุ่น 3B)</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>[gemma3:1b (0.8GB)]: เร็วมาก (130.7 TPS) แต่ในข้อ GT-01 เกิดอาการพูดซ้ำ 'SX1276 Ultrasonic Distance Sensor Module...' และไม่ระบุชื่อโครงงาน The LoRaWAN ทำให้ Phrase Recall ตกเหลือ 33.3%
+[llama3.1:8b (4.9GB)]: ขนาดล้น VRAM 4GB ต้องสลับไปใช้ CPU RAM ทำให้ความเร็วตกเหลือเพียง 7.3 TPS (เฉลี่ย 20.45s/ข้อ)</t>
+        </is>
+      </c>
+      <c r="F10" s="33" t="inlineStr">
+        <is>
+          <t>ตามกฎ Rule 1-7 (Multi-LLM Suitability):
+- `llama3.2:3b` ชนะเลิศความคุ้มค่ารวม (87.70 คะแนน, 5.60s)
+- `qwen2.5:3b` ชนะเลิศความเร็ว 3B (82.48 คะแนน, 60.0 TPS)
+- `gemma3:4b` ชนะเลิศคุณภาพเนื้อหาสูงสุด (Quality 84.67)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="49" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="33" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="33" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="43" customWidth="1" min="19" max="19"/>
+    <col width="52" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>🤖 Stage 3: ตารางเปรียบเทียบโมเดล LLM ทั้ง 7 รุ่น บนการ์ดจอ RTX 3050 Ti (4GB VRAM) + RAM 16GB</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>ล็อกค่าพารามิเตอร์ที่ชนะจาก Stage 1+2 (top_k=15, top_n=10, Chunks=6, Quota=2, Temp=0.0) แล้ววัดคะแนนรายกฎ (Rule 1-7), ความเร็ว และความเหมาะสมกับเครื่อง</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>อันดับ (Rank)</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>ชื่อโมเดล (Ollama Model)</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>ตระกูล (Family)</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>ขนาดพารามิเตอร์</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>ขนาดไฟล์ (GB)</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>ความเข้ากันได้กับ RTX 3050 Ti (4GB VRAM)</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 1: Citation (เต็ม 30)</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 2: Cleanliness (เต็ม 25)</t>
+        </is>
+      </c>
+      <c r="I4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 3: Speed Score (เต็ม 25)</t>
+        </is>
+      </c>
+      <c r="J4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 4: Completeness (เต็ม 20)</t>
+        </is>
+      </c>
+      <c r="K4" s="31" t="inlineStr">
+        <is>
+          <t>รวมคะแนน Rubric (เต็ม 100)</t>
+        </is>
+      </c>
+      <c r="L4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 5: Key Phrase Recall (%)</t>
+        </is>
+      </c>
+      <c r="M4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 6: Hallucination Guard (%)</t>
+        </is>
+      </c>
+      <c r="N4" s="31" t="inlineStr">
+        <is>
+          <t>Multi-Project Coverage (%)</t>
+        </is>
+      </c>
+      <c r="O4" s="31" t="inlineStr">
+        <is>
+          <t>Blended Quality (0-100)</t>
+        </is>
+      </c>
+      <c r="P4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 7: VRAM Fit Score</t>
+        </is>
+      </c>
+      <c r="Q4" s="31" t="inlineStr">
+        <is>
+          <t>เวลาตอบเฉลี่ย (วินาที)</t>
+        </is>
+      </c>
+      <c r="R4" s="31" t="inlineStr">
+        <is>
+          <t>ความเร็ว (TPS)</t>
+        </is>
+      </c>
+      <c r="S4" s="31" t="inlineStr">
+        <is>
+          <t>คะแนนความเหมาะสมรวม (Suitability Score)</t>
+        </is>
+      </c>
+      <c r="T4" s="31" t="inlineStr">
+        <is>
+          <t>คำแนะนำการใช้งาน (Recommendation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>#1</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="inlineStr">
+        <is>
+          <t>llama3.2:3b</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>Meta Llama 3.2</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>3.2B</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="33" t="inlineStr">
+        <is>
+          <t>🟢 100% GPU (เหลือ VRAM 2.0GB)</t>
+        </is>
+      </c>
+      <c r="G5" s="32" t="n">
+        <v>21</v>
+      </c>
+      <c r="H5" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="I5" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="J5" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="K5" s="32" t="n">
+        <v>79</v>
+      </c>
+      <c r="L5" s="32" t="n">
+        <v>86.68000000000001</v>
+      </c>
+      <c r="M5" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="N5" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="O5" s="32" t="n">
+        <v>84.06999999999999</v>
+      </c>
+      <c r="P5" s="32" t="n">
+        <v>97</v>
+      </c>
+      <c r="Q5" s="32" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="R5" s="32" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="S5" s="32" t="n">
+        <v>87.7</v>
+      </c>
+      <c r="T5" s="33" t="inlineStr">
+        <is>
+          <t>🏆 แนะนำอันดับ 1: รุ่นเล็กของ Meta สำหรับ Laptop GPU 4GB (เด่นภาษาอังกฤษ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>#2</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>Alibaba Qwen 2.5</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>3.1B</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F6" s="33" t="inlineStr">
+        <is>
+          <t>🟢 100% GPU (เบาพิเศษ เหลือ VRAM 2.1GB)</t>
+        </is>
+      </c>
+      <c r="G6" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="H6" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="I6" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="J6" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" s="32" t="n">
+        <v>77</v>
+      </c>
+      <c r="L6" s="32" t="n">
+        <v>80.02</v>
+      </c>
+      <c r="M6" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="N6" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="O6" s="32" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="P6" s="32" t="n">
+        <v>98</v>
+      </c>
+      <c r="Q6" s="32" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="R6" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="S6" s="32" t="n">
+        <v>82.48</v>
+      </c>
+      <c r="T6" s="33" t="inlineStr">
+        <is>
+          <t>🏆 แนะนำอันดับ 2: เน้นความเร็วสูงสุดบน RTX 3050 Ti + แม่นคีย์เวิร์ดไทย/อังกฤษ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>#3</t>
+        </is>
+      </c>
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:1b</t>
+        </is>
+      </c>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>Google Gemma 3</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>1.0B</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>🟢 100% GPU (จิ๋วพิเศษ กิน VRAM &lt; 1GB)</t>
+        </is>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>18</v>
+      </c>
+      <c r="H7" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I7" s="35" t="n">
+        <v>16</v>
+      </c>
+      <c r="J7" s="35" t="n">
+        <v>19</v>
+      </c>
+      <c r="K7" s="35" t="n">
+        <v>78</v>
+      </c>
+      <c r="L7" s="35" t="n">
+        <v>66.66</v>
+      </c>
+      <c r="M7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="O7" s="35" t="n">
+        <v>78.47</v>
+      </c>
+      <c r="P7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q7" s="35" t="n">
+        <v>6.86</v>
+      </c>
+      <c r="R7" s="35" t="n">
+        <v>130.7</v>
+      </c>
+      <c r="S7" s="35" t="n">
+        <v>81.31</v>
+      </c>
+      <c r="T7" s="34" t="inlineStr">
+        <is>
+          <t>Ultra-Lightweight ทดสอบขีดจำกัดความเร็วสูงสุดเมื่อลดขนาดเหลือ 1B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:4b</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="inlineStr">
+        <is>
+          <t>Google Gemma 3</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>4.3B</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F8" s="36" t="inlineStr">
+        <is>
+          <t>🟢 100% GPU (พอดี VRAM 4GB)</t>
+        </is>
+      </c>
+      <c r="G8" s="37" t="n">
+        <v>21</v>
+      </c>
+      <c r="H8" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="J8" s="37" t="n">
+        <v>18</v>
+      </c>
+      <c r="K8" s="37" t="n">
+        <v>75</v>
+      </c>
+      <c r="L8" s="37" t="n">
+        <v>86.68000000000001</v>
+      </c>
+      <c r="M8" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="N8" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="O8" s="37" t="n">
+        <v>84.67</v>
+      </c>
+      <c r="P8" s="37" t="n">
+        <v>90</v>
+      </c>
+      <c r="Q8" s="37" t="n">
+        <v>19.23</v>
+      </c>
+      <c r="R8" s="37" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="S8" s="37" t="n">
+        <v>78.03</v>
+      </c>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>Baseline หลัก (สมดุลภาษาไทย-อังกฤษ + โครงสร้าง Markdown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>Alibaba Qwen 2.5</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>7.6B</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Hybrid GPU+CPU (เกิน VRAM 4GB เล็กน้อย)</t>
+        </is>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>24</v>
+      </c>
+      <c r="H9" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>11</v>
+      </c>
+      <c r="J9" s="35" t="n">
+        <v>18</v>
+      </c>
+      <c r="K9" s="35" t="n">
+        <v>78</v>
+      </c>
+      <c r="L9" s="35" t="n">
+        <v>80.02</v>
+      </c>
+      <c r="M9" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N9" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="O9" s="35" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="P9" s="35" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q9" s="35" t="n">
+        <v>16.97</v>
+      </c>
+      <c r="R9" s="35" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="S9" s="35" t="n">
+        <v>74.05</v>
+      </c>
+      <c r="T9" s="34" t="inlineStr">
+        <is>
+          <t>ตัวแทนรุ่นกลาง 7B ความเข้าใจลึกซึ้งแต่ใช้เวลาประมวลผลนานขึ้น</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="C10" s="36" t="inlineStr">
+        <is>
+          <t>Alibaba Qwen 3</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>4.0B</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F10" s="36" t="inlineStr">
+        <is>
+          <t>🟢 100% GPU (เหลือ VRAM 1.5GB)</t>
+        </is>
+      </c>
+      <c r="G10" s="37" t="n">
+        <v>21</v>
+      </c>
+      <c r="H10" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="I10" s="37" t="n">
+        <v>9</v>
+      </c>
+      <c r="J10" s="37" t="n">
+        <v>19</v>
+      </c>
+      <c r="K10" s="37" t="n">
+        <v>74</v>
+      </c>
+      <c r="L10" s="37" t="n">
+        <v>73.34</v>
+      </c>
+      <c r="M10" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="N10" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="O10" s="37" t="n">
+        <v>77.73</v>
+      </c>
+      <c r="P10" s="37" t="n">
+        <v>95</v>
+      </c>
+      <c r="Q10" s="37" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="R10" s="37" t="n">
+        <v>17</v>
+      </c>
+      <c r="S10" s="37" t="n">
+        <v>74</v>
+      </c>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>รุ่นใหม่เน้นการคิดเชิงเหตุผล (Reasoning) และการสกัดข้อมูลเทคนิค</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="35" t="inlineStr">
+        <is>
+          <t>#7</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="C11" s="34" t="inlineStr">
+        <is>
+          <t>Meta Llama 3.1</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>8.0B</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>🟡 Hybrid GPU+CPU (เกิน VRAM 4GB ต้องพึ่ง RAM)</t>
+        </is>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>21</v>
+      </c>
+      <c r="H11" s="35" t="n">
+        <v>23</v>
+      </c>
+      <c r="I11" s="35" t="n">
+        <v>11</v>
+      </c>
+      <c r="J11" s="35" t="n">
+        <v>18</v>
+      </c>
+      <c r="K11" s="35" t="n">
+        <v>73</v>
+      </c>
+      <c r="L11" s="35" t="n">
+        <v>86.68000000000001</v>
+      </c>
+      <c r="M11" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N11" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="O11" s="35" t="n">
+        <v>80.47</v>
+      </c>
+      <c r="P11" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="Q11" s="35" t="n">
+        <v>20.45</v>
+      </c>
+      <c r="R11" s="35" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="S11" s="35" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="T11" s="34" t="inlineStr">
+        <is>
+          <t>ตัวแทนรุ่นใหญ่ 8B มาตรฐานของ Meta</t>
         </is>
       </c>
     </row>
@@ -24245,6 +25551,2235 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="56" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="29" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="35" customWidth="1" min="12" max="12"/>
+    <col width="27" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="56" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>📑 Stage 3 Per-Query Detail: คะแนนแยกตามกฎ (Rule 1-6) และตัวอย่างคำตอบจริงของโมเดล LLM ทั้ง 7 รุ่น</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบคำตอบจริงและคะแนนรายกฎของแต่ละโมเดลในคำถามชุดเดียวกัน (GT-01, GT-03, GT-04, GT-06, GT-08)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>ชื่อโมเดล (Model)</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>ขนาด (GB)</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>รหัสข้อ (Query ID)</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>หมวดหมู่ (Category)</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>คำถามที่ใช้ทดสอบ (Query)</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 1: Citation (30)</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 2: Cleanliness (25)</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 3: Latency (25)</t>
+        </is>
+      </c>
+      <c r="I4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 4: Completeness (20)</t>
+        </is>
+      </c>
+      <c r="J4" s="31" t="inlineStr">
+        <is>
+          <t>Rubric Total (100)</t>
+        </is>
+      </c>
+      <c r="K4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 5: Phrase Recall (%)</t>
+        </is>
+      </c>
+      <c r="L4" s="31" t="inlineStr">
+        <is>
+          <t>Rule 6: Hallucination Guard (%)</t>
+        </is>
+      </c>
+      <c r="M4" s="31" t="inlineStr">
+        <is>
+          <t>Blended Quality (0-100)</t>
+        </is>
+      </c>
+      <c r="N4" s="31" t="inlineStr">
+        <is>
+          <t>เวลา LLM ตอบ (s)</t>
+        </is>
+      </c>
+      <c r="O4" s="31" t="inlineStr">
+        <is>
+          <t>ความเร็ว (TPS)</t>
+        </is>
+      </c>
+      <c r="P4" s="31" t="inlineStr">
+        <is>
+          <t>ตัวอย่างคำตอบจริงจากโมเดล (Actual Model Output Preview)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>llama3.2:3b</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H5" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J5" s="35" t="n">
+        <v>80</v>
+      </c>
+      <c r="K5" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M5" s="35" t="n">
+        <v>88</v>
+      </c>
+      <c r="N5" s="35" t="n">
+        <v>13.23</v>
+      </c>
+      <c r="O5" s="35" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="P5" s="34" t="inlineStr">
+        <is>
+          <t>1. **The LoRaWAN** ([2020]) - โมดูล SX1276 เป็นโมดูลที่ใช้ในการสื่อสารไร้สายสำหรับ LoRaWAN โมดูลนี้มีความสามารถในการส่งและรับข้อมูลได้ไกลถึง 5 กิโลเมตร โดยใช้ความชัน 920-925 MHz [Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>llama3.2:3b</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D6" s="36" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E6" s="36" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F6" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H6" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J6" s="37" t="n">
+        <v>70</v>
+      </c>
+      <c r="K6" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L6" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M6" s="37" t="n">
+        <v>73.67</v>
+      </c>
+      <c r="N6" s="37" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="O6" s="37" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="P6" s="36" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน เป้าหมายหลักของโครงการ LoRaWAN คือการสำรวจฟังก์ชันของเทคโนโลยี LoRaWAN โดยใช้บอร์ด TTGO และ ESP32 เพื่อสร้างระบบสื่อสารที่มีพลังงานต่ำสามารถส่งข้อมูลไปไกลได้โดยไม่ต้องใช้ Bluetooth หรือ Wi-Fi  ### 🏗️ ส่วนประกอบและควา</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="34" t="inlineStr">
+        <is>
+          <t>llama3.2:3b</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D7" s="34" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F7" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G7" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H7" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I7" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="K7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M7" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N7" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - **เอกสารอ้างอิง**: 📄 </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>llama3.2:3b</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H8" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="37" t="n">
+        <v>70</v>
+      </c>
+      <c r="K8" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L8" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M8" s="37" t="n">
+        <v>73.67</v>
+      </c>
+      <c r="N8" s="37" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="O8" s="37" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="P8" s="36" t="inlineStr">
+        <is>
+          <t>ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="34" t="inlineStr">
+        <is>
+          <t>llama3.2:3b</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D9" s="34" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E9" s="34" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F9" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H9" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J9" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="K9" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L9" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M9" s="35" t="n">
+        <v>85</v>
+      </c>
+      <c r="N9" s="35" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="O9" s="35" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="P9" s="34" t="inlineStr">
+        <is>
+          <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | เทคโนโลยีฮาร์ดแวร์ | LoRaWAN, TTGO, ESP32 | ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร |  ## Key Differences - ไม่มีข้อมูลที่เกี่ยวข้องในเอกสารเกี่ยวกั</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H10" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K10" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L10" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M10" s="37" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="N10" s="37" t="n">
+        <v>36.84</v>
+      </c>
+      <c r="O10" s="37" t="n">
+        <v>9</v>
+      </c>
+      <c r="P10" s="36" t="inlineStr">
+        <is>
+          <t>1. **The LoRaWAN** (2020) - โครงงานนี้ใช้โมดูล LoRaWAN และโมดูล TTGO และ ESP32 เพื่อศึกษาการทำงานของเทคโนโลยี LoRaWAN โดยใช้ชิปเซ็ต LoRaWAN และโมดูล TTGO และ ESP32.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b</t>
+        </is>
+      </c>
+      <c r="B11" s="35" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F11" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H11" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="I11" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J11" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="K11" s="35" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L11" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M11" s="35" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="N11" s="35" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="O11" s="35" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="P11" s="34" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน โครงงานนี้มุ่งเน้นในการศึกษาการทำงานของเทคโนโลยี LoRaWAN โดยใช้ชุดอุปกรณ์ TTGO และ ESP32, โดยเฉพาะการสร้างระบบสื่อสารแบบต่ำพลังงานที่สามารถส่งข้อมูลได้หลายกิโลเมตรโดยไม่ต้อง依靠 Bluetooth หรือ Wi-Fi.  ### 🏗️ สถาปัตยกรร</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b</t>
+        </is>
+      </c>
+      <c r="B12" s="37" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D12" s="36" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="G12" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H12" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="I12" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J12" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="K12" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="L12" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M12" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="N12" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - **เอกสารอ้างอิง**: 📄 </t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b</t>
+        </is>
+      </c>
+      <c r="B13" s="35" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C13" s="35" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F13" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G13" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H13" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="J13" s="35" t="n">
+        <v>70</v>
+      </c>
+      <c r="K13" s="35" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L13" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M13" s="35" t="n">
+        <v>73.67</v>
+      </c>
+      <c r="N13" s="35" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="O13" s="35" t="n">
+        <v>79</v>
+      </c>
+      <c r="P13" s="34" t="inlineStr">
+        <is>
+          <t>ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36" t="inlineStr">
+        <is>
+          <t>qwen2.5:3b</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D14" s="36" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E14" s="36" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F14" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G14" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H14" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="I14" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J14" s="37" t="n">
+        <v>75</v>
+      </c>
+      <c r="K14" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="L14" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M14" s="37" t="n">
+        <v>85</v>
+      </c>
+      <c r="N14" s="37" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="O14" s="37" t="n">
+        <v>76</v>
+      </c>
+      <c r="P14" s="36" t="inlineStr">
+        <is>
+          <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | Purpose &amp; Scope | โครงงานนี้ investigates the functionality of LoRaWAN technology using TTGO และ ESP32 บอร์ด, ความสนใจหลักคือการสร้างระบบสื่อ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:1b</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C15" s="35" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D15" s="34" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E15" s="34" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F15" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H15" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J15" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="K15" s="35" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="L15" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M15" s="35" t="n">
+        <v>62.33</v>
+      </c>
+      <c r="N15" s="35" t="n">
+        <v>23.73</v>
+      </c>
+      <c r="O15" s="35" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="P15" s="34" t="inlineStr">
+        <is>
+          <t>1. **SX1276 Ultrasonic Distance Sensor Module:** สามารถวัดระยะทางได้ 2. **SX1276 Ultrasonic Distance Sensor Module:** สามารถวัดระยะทางได้ 3. **SX1276 Ultrasonic Distance Sensor Module:** สามารถวัดระยะทางได้ 4. **SX1276 Ultrasonic Distance S</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:1b</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D16" s="36" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E16" s="36" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F16" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G16" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H16" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="I16" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J16" s="37" t="n">
+        <v>75</v>
+      </c>
+      <c r="K16" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L16" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M16" s="37" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="N16" s="37" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="O16" s="37" t="n">
+        <v>136.4</v>
+      </c>
+      <c r="P16" s="36" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน The LoRaWAN เป็นโครงการวิจัยที่มุ่งเน้นการพัฒนาระบบสื่อสารแบบ LoRaWAN (Long Range Wide Area Network) โดยใช้ TTGO และ ESP32 เพื่อส่งข้อมูลผ่านระยะทางไกลโดยไม่ต้องพึ่งพา Bluetooth หรือ Wi-Fi  โครงการนี้มีเป้าหมายหลักคื</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:1b</t>
+        </is>
+      </c>
+      <c r="B17" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E17" s="34" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F17" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G17" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H17" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I17" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J17" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="K17" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L17" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M17" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N17" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - **เอกสารอ้างอิง**: 📄 </t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:1b</t>
+        </is>
+      </c>
+      <c r="B18" s="37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E18" s="36" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F18" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G18" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H18" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="I18" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="J18" s="37" t="n">
+        <v>75</v>
+      </c>
+      <c r="K18" s="37" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="L18" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M18" s="37" t="n">
+        <v>68.33</v>
+      </c>
+      <c r="N18" s="37" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="O18" s="37" t="n">
+        <v>130.6</v>
+      </c>
+      <c r="P18" s="36" t="inlineStr">
+        <is>
+          <t>The retrieved document does not provide information about the use of Line Notify.  Not specified in the retrieved document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:1b</t>
+        </is>
+      </c>
+      <c r="B19" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C19" s="35" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E19" s="34" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F19" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H19" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="I19" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J19" s="35" t="n">
+        <v>75</v>
+      </c>
+      <c r="K19" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L19" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M19" s="35" t="n">
+        <v>85</v>
+      </c>
+      <c r="N19" s="35" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="O19" s="35" t="n">
+        <v>135.8</v>
+      </c>
+      <c r="P19" s="34" t="inlineStr">
+        <is>
+          <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | Purpose &amp; Scope | Investigating LoRaWAN technology using TTGO and ESP32 boards, focusing on low-power communication. | Designed to locate bea</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:4b</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E20" s="36" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F20" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H20" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J20" s="37" t="n">
+        <v>80</v>
+      </c>
+      <c r="K20" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L20" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M20" s="37" t="n">
+        <v>79.67</v>
+      </c>
+      <c r="N20" s="37" t="n">
+        <v>28.79</v>
+      </c>
+      <c r="O20" s="37" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P20" s="36" t="inlineStr">
+        <is>
+          <t>1. **The LoRaWAN** ([Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18]) ระบุว่า LoRa Implements a physical layer module, which is suitable for P2P applications, without encryption, broadcast data, and if someon</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:4b</t>
+        </is>
+      </c>
+      <c r="B21" s="35" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C21" s="35" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D21" s="34" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E21" s="34" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F21" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G21" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H21" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J21" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="K21" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L21" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M21" s="35" t="n">
+        <v>82</v>
+      </c>
+      <c r="N21" s="35" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="O21" s="35" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="P21" s="34" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน โครงงาน The LoRaWAN มีวัตถุประสงค์เพื่อศึกษาการทำงานของเทคโนโลยี LoRaWAN โดยใช้บอร์ด TTGO และ ESP32 เพื่อสร้างระบบสื่อสารแบบ Low-Power ที่สามารถส่งข้อมูลได้ในระยะหลายกิโลเมตร โดยไม่ต้องใช้ Bluetoo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:4b</t>
+        </is>
+      </c>
+      <c r="B22" s="37" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C22" s="37" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D22" s="36" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E22" s="36" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F22" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="G22" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H22" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="I22" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J22" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="K22" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="L22" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M22" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="N22" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="36" t="inlineStr">
+        <is>
+          <t>อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - *</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="34" t="inlineStr">
+        <is>
+          <t>gemma3:4b</t>
+        </is>
+      </c>
+      <c r="B23" s="35" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D23" s="34" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E23" s="34" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F23" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G23" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H23" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="I23" s="35" t="n">
+        <v>10</v>
+      </c>
+      <c r="J23" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="K23" s="35" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L23" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M23" s="35" t="n">
+        <v>79.67</v>
+      </c>
+      <c r="N23" s="35" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="O23" s="35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P23" s="34" t="inlineStr">
+        <is>
+          <t>ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t>gemma3:4b</t>
+        </is>
+      </c>
+      <c r="B24" s="37" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="C24" s="37" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D24" s="36" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E24" s="36" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G24" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H24" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I24" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J24" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K24" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="L24" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M24" s="37" t="n">
+        <v>82</v>
+      </c>
+      <c r="N24" s="37" t="n">
+        <v>30.92</v>
+      </c>
+      <c r="O24" s="37" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="P24" s="36" t="inlineStr">
+        <is>
+          <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | Purpose &amp; Scope | Establishing a low-power communication system capable of transmitting data over several kilometers with</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D25" s="34" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E25" s="34" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F25" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G25" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H25" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I25" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J25" s="35" t="n">
+        <v>80</v>
+      </c>
+      <c r="K25" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L25" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M25" s="35" t="n">
+        <v>88</v>
+      </c>
+      <c r="N25" s="35" t="n">
+        <v>33.57</v>
+      </c>
+      <c r="O25" s="35" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="P25" s="34" t="inlineStr">
+        <is>
+          <t>1. **โครงงาน The LoRaWAN** ([2020]) - โครงการนี้ศึกษาฟังก์ชันของเทคโนโลยี LoRaWAN ด้วยการใช้ TTGO และ ESP32 บอร์ด ซึ่งโมดูล SX1276 ถูกกล่าวถึงในส่วนของ LoRa ที่ใช้ในโปรเจค [Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 18].</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b</t>
+        </is>
+      </c>
+      <c r="B26" s="37" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C26" s="37" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E26" s="36" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F26" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H26" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I26" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J26" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K26" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L26" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M26" s="37" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="N26" s="37" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="O26" s="37" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="P26" s="36" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน โครงงานนี้ศึกษาฟังก์ชันของเทคโนโลยี LoRaWAN โดยใช้ TTGO และ ESP32 ซึ่งมุ่งเน้นการสร้างระบบการสื่อสารแบบต่ำพลังงานที่สามารถส่งข้อมูลได้หลายกิโลเมตรโดยไม่ต้องพึ่งพา Bluetooth หรือ Wi-Fi.  ### 🏗️ 体系结构 ไม่พบข้อมูลที่เกี่</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b</t>
+        </is>
+      </c>
+      <c r="B27" s="35" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C27" s="35" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D27" s="34" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E27" s="34" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F27" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G27" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H27" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I27" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J27" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="K27" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L27" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M27" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N27" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - **เอกสารอ้างอิง**: 📄 </t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C28" s="37" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D28" s="36" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E28" s="36" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F28" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G28" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H28" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="I28" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="J28" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K28" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L28" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M28" s="37" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="N28" s="37" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="O28" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="P28" s="36" t="inlineStr">
+        <is>
+          <t>ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="34" t="inlineStr">
+        <is>
+          <t>qwen2.5:7b</t>
+        </is>
+      </c>
+      <c r="B29" s="35" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C29" s="35" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D29" s="34" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E29" s="34" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F29" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G29" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H29" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J29" s="35" t="n">
+        <v>80</v>
+      </c>
+      <c r="K29" s="35" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L29" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M29" s="35" t="n">
+        <v>79.67</v>
+      </c>
+      <c r="N29" s="35" t="n">
+        <v>22.97</v>
+      </c>
+      <c r="O29" s="35" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P29" s="34" t="inlineStr">
+        <is>
+          <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | Technologies &amp; Hardware | ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร | Not specified in the retrieved document |  ## Key Differences - ไม่พบข้อมูลที่เก</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="B30" s="37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C30" s="37" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D30" s="36" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E30" s="36" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F30" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G30" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H30" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I30" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J30" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K30" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="L30" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M30" s="37" t="n">
+        <v>79</v>
+      </c>
+      <c r="N30" s="37" t="n">
+        <v>48.95</v>
+      </c>
+      <c r="O30" s="37" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="P30" s="36" t="inlineStr">
+        <is>
+          <t>1. **เข้าใจคำถาม**: ผู้ใช้ถามว่า "โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง" ซึ่งแปลว่า "โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง" หรือ "มีโครงงานอะไรที่ใช้โมดูล SX1276"  2. **วิเคราะห์บริบทที่ได้รับ**: ต้องตรวจสอบเอกสารทั้งหมดที่ให้มาเพื่อหาโครงงาน</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="34" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C31" s="35" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D31" s="34" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E31" s="34" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F31" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G31" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H31" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I31" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J31" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="K31" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L31" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M31" s="35" t="n">
+        <v>79</v>
+      </c>
+      <c r="N31" s="35" t="n">
+        <v>14.55</v>
+      </c>
+      <c r="O31" s="35" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="P31" s="34" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน ขั้นตอนการทำงานและการทดลองของ The LoRaWAN ถูกอธิบายในเอกสารว่าเป็นโครงการวิจัยที่ศึกษาฟังก์ชันการทำงานของเทคโนโลยี LoRaWAN โดยใช้ชิ้นส่วน TTGO และ ESP32 สำหรับการสร้างระบบสื่อสารแบบต่ำพลังงาน สามารถส่งข้อมูลได้ระยะทา</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="36" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="B32" s="37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C32" s="37" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D32" s="36" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E32" s="36" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F32" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="G32" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="I32" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J32" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="K32" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="L32" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M32" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="N32" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - **เอกสารอ้างอิง**: 📄 </t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="34" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="B33" s="35" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C33" s="35" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D33" s="34" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E33" s="34" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F33" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G33" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H33" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I33" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="J33" s="35" t="n">
+        <v>60</v>
+      </c>
+      <c r="K33" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M33" s="35" t="n">
+        <v>51</v>
+      </c>
+      <c r="N33" s="35" t="n">
+        <v>12.85</v>
+      </c>
+      <c r="O33" s="35" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="P33" s="34" t="inlineStr">
+        <is>
+          <t>Okay, let's tackle this question. The user is asking if the project "The LoRaWAN" connects with Line Notify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="36" t="inlineStr">
+        <is>
+          <t>qwen3:4b</t>
+        </is>
+      </c>
+      <c r="B34" s="37" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C34" s="37" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D34" s="36" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E34" s="36" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F34" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="G34" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H34" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I34" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J34" s="37" t="n">
+        <v>80</v>
+      </c>
+      <c r="K34" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L34" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M34" s="37" t="n">
+        <v>79.67</v>
+      </c>
+      <c r="N34" s="37" t="n">
+        <v>14.63</v>
+      </c>
+      <c r="O34" s="37" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="P34" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | Purpose &amp; Scope | Documented Purpose [Source: 1_6031501044_6031501061_FinalProject.pdf, Page: 5] | Not specified in the retrieved document | </t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="inlineStr">
+        <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C35" s="35" t="inlineStr">
+        <is>
+          <t>GT-01</t>
+        </is>
+      </c>
+      <c r="D35" s="34" t="inlineStr">
+        <is>
+          <t>Exact Hardware</t>
+        </is>
+      </c>
+      <c r="E35" s="34" t="inlineStr">
+        <is>
+          <t>โครงงานที่ใช้โมดูล SX1276 มีอะไรบ้าง</t>
+        </is>
+      </c>
+      <c r="F35" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G35" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H35" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I35" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J35" s="35" t="n">
+        <v>80</v>
+      </c>
+      <c r="K35" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L35" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M35" s="35" t="n">
+        <v>88</v>
+      </c>
+      <c r="N35" s="35" t="n">
+        <v>43.81</v>
+      </c>
+      <c r="O35" s="35" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="P35" s="34" t="inlineStr">
+        <is>
+          <t>1. **The LoRaWAN** (2020) - โครงการนี้มุ่งเน้นการสำรวจความสามารถของเทคโนโลยี LoRaWAN โดยใช้บอร์ด TTGO และ ESP32 เพื่อสร้างระบบการสื่อสารที่มีพลังงานต่ำ สามารถส่งสัญญาณข้อมูลได้หลายกิโลเมตรโดยไม่ต้องใช้บลูทูธหรือ Wi-Fi [Source: 1_6031501044_</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="36" t="inlineStr">
+        <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="B36" s="37" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C36" s="37" t="inlineStr">
+        <is>
+          <t>GT-03</t>
+        </is>
+      </c>
+      <c r="D36" s="36" t="inlineStr">
+        <is>
+          <t>Deep Dive Methodology</t>
+        </is>
+      </c>
+      <c r="E36" s="36" t="inlineStr">
+        <is>
+          <t>ขั้นตอนการทำงานและการทดลองของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F36" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G36" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H36" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="I36" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="J36" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K36" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L36" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M36" s="37" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="N36" s="37" t="n">
+        <v>28.22</v>
+      </c>
+      <c r="O36" s="37" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="P36" s="36" t="inlineStr">
+        <is>
+          <t>### 📌 สรุปภาพรวมโครงงาน โครงงาน The LoRaWAN มีวัตถุประสงค์เพื่อศึกษาคุณสมบัติของเทคโนโลยี LoRaWAN โดยใช้บอร์ด TTGO และ ESP32 โดยมุ่งเน้นการสร้างระบบการสื่อสารที่มีความรุนแรงต่ำสามารถส่งสัญญาณข้อมูลได้ไกลหลายกิโลเมตรโดยไม่ต้องใช้บลูทูธหรือ W</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="34" t="inlineStr">
+        <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
+          <t>GT-04</t>
+        </is>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>Fast-Path Metadata</t>
+        </is>
+      </c>
+      <c r="E37" s="34" t="inlineStr">
+        <is>
+          <t>ใครเป็นที่ปรึกษาของ The LoRaWAN</t>
+        </is>
+      </c>
+      <c r="F37" s="35" t="n">
+        <v>30</v>
+      </c>
+      <c r="G37" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="H37" s="35" t="n">
+        <v>25</v>
+      </c>
+      <c r="I37" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J37" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="K37" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L37" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M37" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="N37" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">อาจารย์ที่ปรึกษาของโครงงาน **The LoRaWAN** คือ **Asst. Prof. Dr. Suppakarn Chansareewittaya** ครับ  - **คณะกรรมการตรวจโครงงาน (Committee)**: Dr. Mahamah Sebakor, Dr. Surapong Uttama - **ปีการศึกษา**: 2020 (พ.ศ. 2563) - **เอกสารอ้างอิง**: 📄 </t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="36" t="inlineStr">
+        <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="B38" s="37" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C38" s="37" t="inlineStr">
+        <is>
+          <t>GT-06</t>
+        </is>
+      </c>
+      <c r="D38" s="36" t="inlineStr">
+        <is>
+          <t>Anti-Hallucination Negative</t>
+        </is>
+      </c>
+      <c r="E38" s="36" t="inlineStr">
+        <is>
+          <t>โครงงาน The LoRaWAN มีการเชื่อมต่อกับ Line Notify หรือไม่</t>
+        </is>
+      </c>
+      <c r="F38" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="G38" s="37" t="n">
+        <v>25</v>
+      </c>
+      <c r="H38" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="I38" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="J38" s="37" t="n">
+        <v>65</v>
+      </c>
+      <c r="K38" s="37" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L38" s="37" t="n">
+        <v>100</v>
+      </c>
+      <c r="M38" s="37" t="n">
+        <v>70.67</v>
+      </c>
+      <c r="N38" s="37" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="O38" s="37" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="P38" s="36" t="inlineStr">
+        <is>
+          <t>ไม่พบข้อมูลที่เกี่ยวข้องในเอกสาร</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>llama3.1:8b</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="C39" s="35" t="inlineStr">
+        <is>
+          <t>GT-08</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>Multi-Project Comparison</t>
+        </is>
+      </c>
+      <c r="E39" s="34" t="inlineStr">
+        <is>
+          <t>เปรียบเทียบโครงงาน The LoRaWAN กับโครงงาน Beacon Signal Location Device ในด้านฮาร์ดแวร์</t>
+        </is>
+      </c>
+      <c r="F39" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="G39" s="35" t="n">
+        <v>15</v>
+      </c>
+      <c r="H39" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="I39" s="35" t="n">
+        <v>20</v>
+      </c>
+      <c r="J39" s="35" t="n">
+        <v>55</v>
+      </c>
+      <c r="K39" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="L39" s="35" t="n">
+        <v>100</v>
+      </c>
+      <c r="M39" s="35" t="n">
+        <v>73</v>
+      </c>
+      <c r="N39" s="35" t="n">
+        <v>25.17</v>
+      </c>
+      <c r="O39" s="35" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="P39" s="34" t="inlineStr">
+        <is>
+          <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | ฮาร์ดแวร์ | TTGO และ ESP32 | ไม่ระบุ |  ## Key Differences - ฮาร์ดแวร์ที่ใช้ของ The LoRaWAN คือ TTGO และ ESP32 ในขณะที่ไม่ระบุฮาร์ดแวร์ที่ใช้</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
docs(eval): add explicit Why-Tested and Why-Selected rationale columns across Stage 1, 2, and Multi-LLM Excel sheets
</commit_message>
<xml_diff>
--- a/backend/data/RAGcoon_Handoff_Specification.xlsx
+++ b/backend/data/RAGcoon_Handoff_Specification.xlsx
@@ -964,15 +964,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="47" customWidth="1" min="2" max="2"/>
     <col width="47" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -998,7 +999,7 @@
       </c>
       <c r="B4" s="31" t="inlineStr">
         <is>
-          <t>ชื่อพารามิเตอร์ (Parameter)</t>
+          <t>ชื่อพารามิเตอร์ / โมเดล (Parameter / Model)</t>
         </is>
       </c>
       <c r="C4" s="31" t="inlineStr">
@@ -1008,17 +1009,22 @@
       </c>
       <c r="D4" s="31" t="inlineStr">
         <is>
-          <t>ช่วงค่าที่ทดสอบทั้งหมด (Tested Range)</t>
+          <t>ช่วงค่าที่นำมาทดสอบ (Tested Range)</t>
         </is>
       </c>
       <c r="E4" s="31" t="inlineStr">
         <is>
-          <t>ค่าที่ดีที่สุด (Optimal Value)</t>
+          <t>ค่าที่เลือกใช้ (Selected Winner)</t>
         </is>
       </c>
       <c r="F4" s="31" t="inlineStr">
         <is>
-          <t>เหตุผลและผลลัพธ์จากการทดลองจริง (Empirical Justification)</t>
+          <t>ทำไมถึงนำมาทดสอบ (Why Tested / สมมติฐานการทดลอง)</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงเลือกค่านี้เป็นผู้ชนะ (Why Selected / เหตุผลเชิงประจักษ์)</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1052,12 @@
       </c>
       <c r="F5" s="33" t="inlineStr">
         <is>
-          <t>ชนะใน Exp 1 (Composite = 88.15, Hit=92.3%, MRR=0.8718, 468.8ms): ดึง Candidate Pool กว้างพอให้ Reranker คัดเนื้อหาเทคนิคขึ้นอันดับ 1 โดยไม่ช้าเหมือน top_k=100 (1,740ms)</t>
+          <t>เพื่อหาขนาด Candidate Pool เริ่มต้นจาก Qdrant ที่สมดุลที่สุด: หากดึงน้อยเกินไป (เช่น 5) เนื้อหาเทคนิคในบทที่ 3-4 อาจตกหล่นตั้งแต่แรก แต่หากดึงมากเกินไป (เช่น 50-100) จะเกิดความหน่วงและมีเอกสารที่ไม่เกี่ยวข้องปะปนเข้ามามาก</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>เลือก top_k = 15 เพราะชนะเลิศใน Exp 1 (Composite = 88.15, Hit=92.3%, MRR=0.8718, ใช้เวลาเพียง 468.8ms): กว้างพอให้ Reranker ดึงเนื้อหาเทคนิคขึ้นอันดับ 1 ได้ครบถ้วน และเร็วกว่า top_k=100 (1,740.7ms) ถึง 3.7 เท่า</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1085,12 @@
       </c>
       <c r="F6" s="33" t="inlineStr">
         <is>
-          <t>ชนะใน Exp 2 (Best Cutoff = 10, Composite = 90.05, Hit=100%, MRR=0.8795): สมดุลระหว่าง Recall@N (96.2%) และ Precision@N (75.6%) ก่อนส่งเข้า Context Assembly</t>
+          <t>เพื่อหาจุดตัด (Cutoff) หลังผ่าน Cross-Encoder Reranker ว่าควรคัดไว้กี่ Chunks ก่อนส่งไปจัดโควตาเข้า LLM: หากคัดน้อยเกินไป (1-3) จะไม่พอสำหรับคำถามเปรียบเทียบหลายโปรเจกต์ แต่หากคัดมากเกินไป (15-30) Precision@N จะลดลง</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>เลือก rerank_top_n = 10 (และใช้คู่กับ Context Cap = 6) เพราะชนะเลิศใน Exp 2 (Composite = 90.05, Hit Rate = 100.0%, MRR = 0.8795, Recall@N = 96.2%) ทำให้ไม่พลาดเอกสารในคำถามเปรียบเทียบหลายโครงงาน</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1110,7 @@
       </c>
       <c r="D7" s="32" t="inlineStr">
         <is>
-          <t>[True (BM25+E5), False (Dense Only)]</t>
+          <t>[True (BM25+E5), False (Dense Only), BM25 Only]</t>
         </is>
       </c>
       <c r="E7" s="32" t="inlineStr">
@@ -1104,7 +1120,12 @@
       </c>
       <c r="F7" s="33" t="inlineStr">
         <is>
-          <t>เปิด Hybrid RRF (BM25 + Multilingual-E5) ดัน Hit Rate เป็น 100% และ MRR 0.9231 (หากปิดเหลือแต่ Dense คะแนน MRR ตกเหลือ 0.7769 เพราะพลาดรหัสชิป SX1276/BLE)</t>
+          <t>เพื่อพิสูจน์ว่าการใช้เฉพาะเวกเตอร์ความหมาย (Dense E5) หรือใช้เฉพาะคำค้น (BM25) อย่างใดอย่างหนึ่ง เพียงพอต่อการค้นหารหัสชิปฮาร์ดแวร์ (SX1276, ESP32) และชื่อเฉพาะของโครงงานหรือไม่</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>เลือกเปิด Hybrid RRF (True) เพราะดัน Hit Rate เต็ม 100.0% และ MRR = 0.9231 ในขณะที่เมื่อปิดเหลือแต่ Dense Only คะแนน Hit Rate ตกเหลือ 84.6% และ MRR ตกเหลือ 0.7769 เพราะเวกเตอร์จับรหัสชิปเฉพาะทางพลาด</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1155,12 @@
       </c>
       <c r="F8" s="33" t="inlineStr">
         <is>
-          <t>เปิด BGE Cross-Encoder Reranker ดัน MRR จาก 0.7436 ขึ้นเป็น 0.9231 (+18.0%) เพราะจัดลำดับย่อหน้าที่มีคำตอบจริงขึ้นเป็น Rank #1</t>
+          <t>เพื่อพิสูจน์ว่าลำดับคะแนนดิบจาก RRF (Vector+BM25) เพียงพอหรือไม่ หรือจำเป็นต้องใช้โมเดล BGE Cross-Encoder Reranker มาอ่านเทียบคู่ (Query, Chunk) ซ้ำอีกครั้ง</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>เลือกเปิด Reranker (True) เพราะช่วยดัน MRR จาก 0.7436 พุ่งขึ้นเป็น 0.9231 (+18.0%) โดยดันย่อหน้าที่มีคำตอบเทคนิคจริงขึ้นเป็นอันดับ 1 (Rank #1) แทนที่หน้าบทนำทั่วไป</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1190,12 @@
       </c>
       <c r="F9" s="33" t="inlineStr">
         <is>
-          <t>เปิดกรองขยะเอกสาร (สารบัญ, กิตติกรรมประกาศ, บรรณานุกรม, ลายเซ็น) ลด Noise Rate จาก 25.0% เหลือ 0.0%</t>
+          <t>เพื่อทดสอบผลกระทบของหน้าขยะในเล่มปริญญานิพนธ์ (เช่น สารบัญ, กิตติกรรมประกาศ, บรรณานุกรม, ใบรับรองลายเซ็น) ที่มักมีคีย์เวิร์ดซ้ำกับคำถามและชอบแย่งพื้นที่ Top-N</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>เลือกเปิด Boilerplate Filter (True) เพราะขจัดขยะเอกสารออกได้ 100% (Noise Rate ลดจาก 25.0% เหลือ 0.0%) และทำให้ MRR เพิ่มจาก 0.7372 เป็น 0.9231</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1225,12 @@
       </c>
       <c r="F10" s="33" t="inlineStr">
         <is>
-          <t>เปิดทางลัด Metadata Scroll ลดเวลาค้นหาเฉลี่ยจาก 555.8ms เหลือ 312.4ms และตอบคำถามอาจารย์/ผู้จัดทำได้ใน 0.01 วินาที</t>
+          <t>เพื่อทดสอบว่าคำถามที่ถามข้อมูลโครงสร้าง (เช่น อาจารย์ที่ปรึกษา, ผู้จัดทำ, ปีการศึกษา) ควรดึงผ่าน Metadata Scroll โดยตรงแทนการค้นหาเวกเตอร์และรอ LLM หรือไม่</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>เลือกเปิด Fast-Path (True) เพราะลดเวลาค้นหาเฉลี่ยทั้งระบบจาก 555.8ms เหลือ 312.4ms และตอบคำถามหมวดอาจารย์ที่ปรึกษา (GT-04) ได้ถูกต้อง 100% ในเวลาเพียง 0.24 วินาที</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1258,12 @@
       </c>
       <c r="F11" s="33" t="inlineStr">
         <is>
-          <t>ชนะใน Exp 4 (Chunks=6, Quality=84.7, Phrase Recall=86.7%): ให้บริบทครบถ้วนสำหรับ LLM โดยไม่เปลือง Input Tokens เกินจำเป็น</t>
+          <t>เพื่อหาจำนวน Chunks สูงสุดที่จะส่งเข้า Prompt ของ LLM บนการ์ดจอ VRAM 4GB: หากส่งน้อยเกินไป (2-4 Chunks) ข้อมูลจะไม่ครบ แต่หากส่งมากเกินไป (10-15 Chunks) จะเกิดอาการ Lost-in-the-Middle และกินเวลาประมวลผล Input Tokens นาน</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>เลือก max_context_chunks = 6 เพราะทำคะแนนคุณภาพคำตอบสูงสุด (Quality = 84.67, Key Phrase Recall = 86.7%) โดยใช้ Input Tokens เฉลี่ยเพียง 1,675 tokens เร็วและแม่นยำกว่าการส่ง 10-15 Chunks (Quality 82.4-83.0)</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1291,12 @@
       </c>
       <c r="F12" s="33" t="inlineStr">
         <is>
-          <t>ล็อกโควตา 2 Chunks/โปรเจกต์ ป้องกันปัญหา Context Starvation เวลาเปรียบเทียบหลายโปรเจกต์ (Multi-Project Coverage = 100%)</t>
+          <t>เพื่อแก้ปัญหา Context Starvation ที่โปรเจกต์เดียวที่มีคะแนนเวกเตอร์สูงกว่ากินพื้นที่ Chunks ทั้งหมด จนโปรเจกต์ที่ 2 ไม่ถูกส่งเข้า LLM ในคำถามเปรียบเทียบ (GT-08)</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>เลือกโควตา 2 Chunks/โปรเจกต์ เพราะทำให้แบ่งพื้นที่ 6 Chunks ได้ถึง 3 โปรเจกต์อย่างยุติธรรม ส่งผลให้ Multi-Project Coverage เต็ม 100.0% และมีรายละเอียดเพียงพอต่อการสร้างตารางเปรียบเทียบ</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1326,12 @@
       </c>
       <c r="F13" s="33" t="inlineStr">
         <is>
-          <t>ชนะใน Exp 5 (Composite = 83.50): รูปแบบ Prompt 'deep_academic' และ 'balanced' ให้โครงสร้างคำตอบและการอ้างอิงครบถ้วนที่สุด</t>
+          <t>เพื่อทดสอบว่ารูปแบบคำสั่ง System Prompt แบบใดช่วยให้ LLM เขียนคำตอบภาษาไทย จัดโครงสร้างหัวข้อ และแนบอ้างอิง `[Source: ..., Page: ...]` ได้ตรงตามกฎ Rubric มากที่สุด</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>เลือก 'deep_academic' (ควบคู่กับ 'balanced') เพราะได้คะแนนรวม Stage 2 สูงสุด (83.50) ได้คะแนน Citation เต็มในข้อเนื้อหา และไม่ตัดจบสั้นเกินไปเหมือน 'concise'</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1359,12 @@
       </c>
       <c r="F14" s="33" t="inlineStr">
         <is>
-          <t>Temperature = 0.0 รักษาความแม่นยำตามเอกสารอ้างอิง 100% (Deterministic Grounding) และเร็วกว่า Temp 0.2/0.5</t>
+          <t>เพื่อพิสูจน์ว่างานถาม-ตอบเอกสารวิชาการ (Academic RAG) ควรเปิดให้โมเดลสุ่มคำศัพท์ (Temp &gt; 0) หรือควรล็อกการตัดสินใจแบบ Deterministic (Temp = 0.0) เพื่อป้องกันอาการมั่วข้อมูล (Hallucination)</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>เลือก temperature = 0.0 เพราะให้ผลลัพธ์เที่ยงตรง 100% (Reproducible), ผ่านกฎ Anti-Hallucination Guard 100.0% และตอบได้เร็วกว่า Temp 0.2 และ 0.5</t>
         </is>
       </c>
     </row>
@@ -1333,12 +1389,17 @@
       </c>
       <c r="E15" s="32" t="inlineStr">
         <is>
-          <t>llama3.2:3b (และ gemma3:4b / qwen2.5:3b)</t>
+          <t>llama3.2:3b (เร็วคุ้มค่า) &amp; gemma3:4b (คุณภาพสูงสุด)</t>
         </is>
       </c>
       <c r="F15" s="33" t="inlineStr">
         <is>
-          <t>ชนะเลิศด้านความคุ้มค่าบน RTX 3050 Ti (4GB VRAM): Suitability Score = 87.70, เวลาตอบเฉลี่ย 5.60s (47.6 TPS)</t>
+          <t>เพื่อค้นหาว่าบนข้อจำกัดฮาร์ดแวร์จริง (RTX 3050 Ti 4GB VRAM + RAM 16GB) โมเดลขนาดใด (1B vs 3B vs 4B vs 7B/8B) ให้จุดสมดุลระหว่างความแม่นยำภาษาไทย การอ้างอิง และความเร็วในการตอบดีที่สุด</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>เลือกใช้งาน 2 โหมดตามจุดประสงค์: (1) llama3.2:3b (2.0GB) ชนะเลิศความคุ้มค่ารวม (Suitability = 87.70, ตอบไว 5.60s / 47.6 TPS, Phrase Recall 86.7%) และ qwen2.5:3b (60.0 TPS) สำหรับเน้นความเร็วสูง (2) gemma3:4b (3.3GB) ชนะเลิศคุณภาพเนื้อหาสูงสุด (Quality = 84.67) สำหรับเน้นภาษาไทยและตารางวิชาการละเอียด</t>
         </is>
       </c>
     </row>
@@ -1353,10 +1414,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -1372,6 +1433,8 @@
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="27" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="52" customWidth="1" min="17" max="17"/>
+    <col width="52" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1470,6 +1533,16 @@
           <t>สถานะ (Status)</t>
         </is>
       </c>
+      <c r="Q4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงนำค่านี้มาทดสอบ (Why Tested)</t>
+        </is>
+      </c>
+      <c r="R4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงเลือก / ไม่เลือกค่านี้ (Why Selected / Verdict)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
@@ -1482,7 +1555,7 @@
           <t>top_k = 100</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="C5" s="35" t="inlineStr">
         <is>
           <t>sweep_topk_100</t>
         </is>
@@ -1528,6 +1601,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q5" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบเพดานสูงสุด (Upper Bound) เมื่อดึง Candidate Pool กว้างสุด 100 ชิ้น</t>
+        </is>
+      </c>
+      <c r="R5" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: ใช้เวลาค้นหาพุ่งถึง 1,740.7 ms (ช้ากว่า top_k=15 ถึง 3.7 เท่า) โดยที่ความแม่นยำไม่ได้เพิ่มขึ้น</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="36" t="inlineStr">
@@ -1540,7 +1623,7 @@
           <t>top_k = 50</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>sweep_topk_50</t>
         </is>
@@ -1586,6 +1669,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q6" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบ Candidate Pool ขนาดใหญ่ (50 ชิ้น) สำหรับคำถามที่คีย์เวิร์ดกระจายหลายหน้า</t>
+        </is>
+      </c>
+      <c r="R6" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: ใช้เวลาค้นหา 977.6 ms ช้าเกินไปเมื่อเทียบกับ top_k=15 ที่ได้ Hit Rate และ MRR เท่ากัน</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="34" t="inlineStr">
@@ -1598,7 +1691,7 @@
           <t>top_k = 30</t>
         </is>
       </c>
-      <c r="C7" s="34" t="inlineStr">
+      <c r="C7" s="35" t="inlineStr">
         <is>
           <t>sweep_topk_30</t>
         </is>
@@ -1644,6 +1737,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q7" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบค่ามาตรฐานเดิมของระบบ (Baseline เดิม = 30 ชิ้น)</t>
+        </is>
+      </c>
+      <c r="R7" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ รองชนะเลิศ: แม่นยำเท่ากับ top_k=15 แต่ใช้เวลาค้นหานานกว่า (675.2 ms vs 468.8 ms)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="33" t="inlineStr">
@@ -1656,7 +1759,7 @@
           <t>top_k = 15</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>sweep_topk_15</t>
         </is>
@@ -1702,6 +1805,16 @@
           <t>🏆 WINNER</t>
         </is>
       </c>
+      <c r="Q8" s="33" t="inlineStr">
+        <is>
+          <t>ทดสอบจุดสมดุล (Sweet Spot = 15 ชิ้น) ระหว่างความเร็วและความครอบคลุมของเนื้อหา</t>
+        </is>
+      </c>
+      <c r="R8" s="33" t="inlineStr">
+        <is>
+          <t>🏆 เลือกเป็นผู้ชนะ (Composite 88.15): ดึงเนื้อหาเทคนิคครบ (Hit 92.3%, MRR 0.8718) และใช้เวลาเพียง 468.8 ms</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="34" t="inlineStr">
@@ -1714,7 +1827,7 @@
           <t>top_k = 10</t>
         </is>
       </c>
-      <c r="C9" s="34" t="inlineStr">
+      <c r="C9" s="35" t="inlineStr">
         <is>
           <t>sweep_topk_10</t>
         </is>
@@ -1760,6 +1873,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q9" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบการลดขนาด Pool ลงเหลือ 10 ชิ้นเพื่อเน้นความเร็วในการค้นหา</t>
+        </is>
+      </c>
+      <c r="R9" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ ไม่เลือก: เร็วขึ้นเล็กน้อย (371.4 ms) แต่เสี่ยงพลาด Chunk ในคำถามที่เอกสารมีหลายบท</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="36" t="inlineStr">
@@ -1772,7 +1895,7 @@
           <t>top_k = 5</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C10" s="37" t="inlineStr">
         <is>
           <t>sweep_topk_5</t>
         </is>
@@ -1818,6 +1941,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q10" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบขีดจำกัดล่าง (Lower Bound = 5 ชิ้น) ดึงเฉพาะ 5 อันดับแรกจาก Qdrant</t>
+        </is>
+      </c>
+      <c r="R10" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: แคบเกินไป! เนื้อหาบทที่ 3-4 หลุดจาก Pool ทำให้ Hit Rate ตกเหลือ 76.9% และ MRR ตกเหลือ 0.5577</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="34" t="inlineStr">
@@ -1830,7 +1963,7 @@
           <t>rerank_top_n = 30</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C11" s="35" t="inlineStr">
         <is>
           <t>sweep_topn_30</t>
         </is>
@@ -1876,6 +2009,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q11" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบการไม่ตัด Chunks ทิ้งหลัง Rerank (ส่งต่อทั้ง 30 ชิ้น)</t>
+        </is>
+      </c>
+      <c r="R11" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: มี Chunks ที่ไม่เกี่ยวข้องปะปนสูง ทำให้ Precision@N ตกเหลือเพียง 53.7%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
@@ -1888,7 +2031,7 @@
           <t>rerank_top_n = 15</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="37" t="inlineStr">
         <is>
           <t>sweep_topn_15</t>
         </is>
@@ -1934,6 +2077,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q12" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบการเก็บ 후보 15 ชิ้นหลัง Rerank เผื่อคำถามเปรียบเทียบหลายโปรเจกต์</t>
+        </is>
+      </c>
+      <c r="R12" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ ไม่เลือก: ได้ Hit Rate 100% แต่ Precision@N (67.1%) ต่ำกว่า rerank_top_n=10</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="33" t="inlineStr">
@@ -1946,7 +2099,7 @@
           <t>rerank_top_n = 10</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>sweep_topn_10</t>
         </is>
@@ -1992,6 +2145,16 @@
           <t>🏆 WINNER</t>
         </is>
       </c>
+      <c r="Q13" s="33" t="inlineStr">
+        <is>
+          <t>ทดสอบจุดสมดุลการคัดกรองหลัง Cross-Encoder Reranker (10 ชิ้น)</t>
+        </is>
+      </c>
+      <c r="R13" s="33" t="inlineStr">
+        <is>
+          <t>🏆 เลือกเป็นผู้ชนะ (Composite 90.05): Hit Rate เต็ม 100.0%, Recall@N สูงถึง 96.2% และ Precision@N สมดุล (75.6%)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="36" t="inlineStr">
@@ -2004,7 +2167,7 @@
           <t>rerank_top_n = 5</t>
         </is>
       </c>
-      <c r="C14" s="36" t="inlineStr">
+      <c r="C14" s="37" t="inlineStr">
         <is>
           <t>sweep_topn_5</t>
         </is>
@@ -2050,6 +2213,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q14" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบการคัดเฉพาะ Top-5 ที่คะแนน Rerank สูงสุด</t>
+        </is>
+      </c>
+      <c r="R14" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ รองชนะเลิศ: แม่นยำสูงในคำถามเดี่ยว แต่ในคำถามเปรียบเทียบหลายโปรเจกต์มีโอกาสที่โปรเจกต์ที่ 2 จะหลุดขอบ</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="34" t="inlineStr">
@@ -2062,7 +2235,7 @@
           <t>rerank_top_n = 3</t>
         </is>
       </c>
-      <c r="C15" s="34" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>sweep_topn_3</t>
         </is>
@@ -2108,6 +2281,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="Q15" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบการคัดแบบเข้มงวดเหลือเพียง 3 ชิ้นแรก</t>
+        </is>
+      </c>
+      <c r="R15" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: แคบเกินไปสำหรับคำถามเชิงลึกและคำถามเปรียบเทียบ (Composite ลดเหลือ 86.26)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
@@ -2120,7 +2303,7 @@
           <t>rerank_top_n = 1</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C16" s="37" t="inlineStr">
         <is>
           <t>sweep_topn_1</t>
         </is>
@@ -2164,6 +2347,16 @@
       <c r="P16" s="37" t="inlineStr">
         <is>
           <t>Tested</t>
+        </is>
+      </c>
+      <c r="Q16" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบสุดโต่ง (Extreme Top-1) คืนเฉพาะ Chunk อันดับ 1 ชิ้นเดียว</t>
+        </is>
+      </c>
+      <c r="R16" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: ตอบคำถามเปรียบเทียบ 2 โครงงาน (GT-08) ไม่ได้เลย เพราะส่งได้แค่โครงงานเดียว (Recall@N ตกเหลือ 80.8%)</t>
         </is>
       </c>
     </row>
@@ -2178,10 +2371,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -2195,7 +2388,8 @@
     <col width="23" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
     <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="48" customWidth="1" min="15" max="15"/>
+    <col width="52" customWidth="1" min="15" max="15"/>
+    <col width="52" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2286,7 +2480,12 @@
       </c>
       <c r="O4" s="31" t="inlineStr">
         <is>
-          <t>ข้อค้นพบจากการเปิด/ปิดโมดูล (Key Takeaway)</t>
+          <t>ทำไมถึงนำมาทดสอบ (Why Tested)</t>
+        </is>
+      </c>
+      <c r="P4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงเลือก / ไม่เลือก (Why Selected &amp; Impact)</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2548,12 @@
       </c>
       <c r="O5" s="33" t="inlineStr">
         <is>
-          <t>เปิดครบทุกโมดูล (Hybrid BM25+E5 + Cross-Encoder Rerank + Boilerplate Filter + Fast-Path)</t>
+          <t>ทดสอบระบบ RAGcoon ที่เปิดครบทุกโมดูล (Hybrid BM25+E5 + Reranker + Filter + Fast-Path) เป็นเกณฑ์มาตรฐานสูงสุด</t>
+        </is>
+      </c>
+      <c r="P5" s="33" t="inlineStr">
+        <is>
+          <t>🏆 เลือกใช้งานจริง (Composite 91.64): Hit Rate เต็ม 100.0%, MRR สูงสุด 0.9231, ขยะเป็น 0.0% และค้นหาเร็วเพียง 312.4 ms</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2616,12 @@
       </c>
       <c r="O6" s="36" t="inlineStr">
         <is>
-          <t>ปิด BM25 ค้นหาเฉพาะเวกเตอร์ E5 (enable_hybrid=False)</t>
+          <t>ทดสอบปิด Sparse BM25 เหลือเฉพาะเวกเตอร์ความหมาย (Multilingual-E5) เพื่อพิสูจน์ว่าเวกเตอร์อย่างเดียวจับรหัสชิปได้หรือไม่</t>
+        </is>
+      </c>
+      <c r="P6" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: เมื่อขาด BM25 ระบบพลาดรหัสฮาร์ดแวร์เฉพาะทาง (SX1276) ทำให้ Hit Rate ตกเหลือ 84.6% และ MRR ตกเหลือ 0.7769</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2684,12 @@
       </c>
       <c r="O7" s="34" t="inlineStr">
         <is>
-          <t>ปิดเวกเตอร์ E5 ค้นหาเฉพาะคีย์เวิร์ด BM25 (enable_bm25_only=True)</t>
+          <t>ทดสอบปิดเวกเตอร์ความหมาย เหลือเฉพาะการค้นหาคำตรงตัว (BM25 Keyword) เพื่อดูว่าค้นหาคำพ้องความหมายได้หรือไม่</t>
+        </is>
+      </c>
+      <c r="P7" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: แม้จับชื่อเฉพาะได้ดี แต่เมื่อคำถามใช้คำอธิบายเชิงความหมายโดยไม่ตรงคีย์เวิร์ดเป๊ะ คะแนน Composite ลดเหลือ 88.24</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2752,12 @@
       </c>
       <c r="O8" s="36" t="inlineStr">
         <is>
-          <t>ปิด Cross-Encoder Reranker ใช้ลำดับจาก RRF โดยตรง (enable_reranker=False)</t>
+          <t>ทดสอบปิด BGE Cross-Encoder Reranker เพื่อดูว่าลำดับคะแนนดิบจาก Qdrant RRF แม่นยำพอสำหรับส่งเข้า LLM หรือยัง</t>
+        </is>
+      </c>
+      <c r="P8" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: เมื่อปิด Reranker ย่อหน้าที่มีคำตอบจริงตกไปอยู่อันดับ 2-4 ทำให้ MRR ร่วงจาก 0.9231 เหลือ 0.7436 (-18.0%)</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2820,12 @@
       </c>
       <c r="O9" s="34" t="inlineStr">
         <is>
-          <t>ปิดตัวกรองขยะเอกสาร สารบัญ/อ้างอิง/ลายเซ็น (enable_boilerplate_filter=False)</t>
+          <t>ทดสอบปิดตัวกรองขยะเอกสาร (Boilerplate Filter) เพื่อดูว่าหน้าสารบัญ/บรรณานุกรม/กิตติกรรมประกาศส่งผลเสียแค่ไหน</t>
+        </is>
+      </c>
+      <c r="P9" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: หน้าสารบัญและกิตติกรรมประกาศหลุดเข้ามาแย่งพื้นที่ Top-N ถึง 25.0% ทำให้ MRR ตกเหลือ 0.7372 (Composite เหลือ 76.26)</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2888,12 @@
       </c>
       <c r="O10" s="36" t="inlineStr">
         <is>
-          <t>ปิดทางลัด Metadata Scroll บังคับรัน Vector+Rerank ทุกข้อ (enable_fast_path=False)</t>
+          <t>ทดสอบปิดทางลัด Metadata Scroll เพื่อดูความแตกต่างของเวลาค้นหาและความแม่นยำในคำถามหมวดอาจารย์ที่ปรึกษา/ผู้จัดทำ</t>
+        </is>
+      </c>
+      <c r="P10" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ ไม่เลือก: ความแม่นยำยังสูงแต่เวลาค้นหาเฉลี่ยช้าลงเกือบเท่าตัว (จาก 312.4 ms เพิ่มเป็น 555.8 ms)</t>
         </is>
       </c>
     </row>
@@ -2728,6 +2957,11 @@
       <c r="O11" s="34" t="inlineStr">
         <is>
           <t>ระบบเก่าดั้งเดิม: Dense ล้วน + ไม่มี Reranker + ไม่มีตัวกรองขยะ + ไม่มี Fast-Path</t>
+        </is>
+      </c>
+      <c r="P11" s="34" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
         </is>
       </c>
     </row>
@@ -2742,11 +2976,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="49" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -2764,6 +2998,8 @@
     <col width="18" customWidth="1" min="17" max="17"/>
     <col width="27" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="52" customWidth="1" min="20" max="20"/>
+    <col width="52" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2877,6 +3113,16 @@
           <t>สถานะ (Status)</t>
         </is>
       </c>
+      <c r="T4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงนำค่านี้มาทดสอบ (Why Tested)</t>
+        </is>
+      </c>
+      <c r="U4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงเลือก / ไม่เลือกค่านี้ (Why Selected / Verdict)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="34" t="inlineStr">
@@ -2889,7 +3135,7 @@
           <t>Chunks=15, Quota=5 (Extra Wide)</t>
         </is>
       </c>
-      <c r="C5" s="34" t="inlineStr">
+      <c r="C5" s="35" t="inlineStr">
         <is>
           <t>sweep_chunks_15_quota_5</t>
         </is>
@@ -2948,6 +3194,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T5" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบเพดานบริบทกว้างสุด (15 Chunks, โควตา 5/โปรเจกต์) เพื่อดูว่ายิ่งส่งเนื้อหาเยอะ LLM ยิ่งตอบดีขึ้นหรือไม่</t>
+        </is>
+      </c>
+      <c r="U5" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: เกิดอาการสำลักบริบท (Context Overload) ในข้อ GT-01 ทำให้ Phrase Recall ตกเหลือ 80.0% และกิน Input Tokens สูงถึง 1,720 tokens</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="36" t="inlineStr">
@@ -2960,7 +3216,7 @@
           <t>Chunks=10, Quota=3 (Wide)</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="37" t="inlineStr">
         <is>
           <t>sweep_chunks_10_quota_3</t>
         </is>
@@ -3019,6 +3275,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T6" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบบริบทขนาดใหญ่ (10 Chunks, โควตา 3/โปรเจกต์)</t>
+        </is>
+      </c>
+      <c r="U6" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: ใช้ Input Tokens เยอะเกินจำเป็น แต่ได้ Key Phrase Recall 80.0% ต่ำกว่าการส่ง 6 Chunks</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="33" t="inlineStr">
@@ -3031,7 +3297,7 @@
           <t>Chunks=6, Quota=2 (Balanced Boost)</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr">
+      <c r="C7" s="32" t="inlineStr">
         <is>
           <t>sweep_chunks_6_quota_2</t>
         </is>
@@ -3090,6 +3356,16 @@
           <t>🏆 WINNER</t>
         </is>
       </c>
+      <c r="T7" s="33" t="inlineStr">
+        <is>
+          <t>ทดสอบจุดสมดุล (6 Chunks, ล็อกโควตา 2 Chunks/โปรเจกต์) เพื่อให้รองรับการเปรียบเทียบ 3 โปรเจกต์อย่างเท่าเทียม</t>
+        </is>
+      </c>
+      <c r="U7" s="33" t="inlineStr">
+        <is>
+          <t>🏆 เลือกเป็นผู้ชนะ Exp 4 (Composite 83.75): ได้ Quality สูงสุด 84.67, Key Phrase Recall สูงสุด 86.68%, และ Multi-Project Coverage เต็ม 100%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="36" t="inlineStr">
@@ -3102,7 +3378,7 @@
           <t>Chunks=5, Quota=2 (Standard Baseline)</t>
         </is>
       </c>
-      <c r="C8" s="36" t="inlineStr">
+      <c r="C8" s="37" t="inlineStr">
         <is>
           <t>sweep_chunks_5_quota_2</t>
         </is>
@@ -3161,6 +3437,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T8" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบค่ามาตรฐานเดิม (5 Chunks, โควตา 2/โปรเจกต์)</t>
+        </is>
+      </c>
+      <c r="U8" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ รองชนะเลิศ: ประสิทธิภาพใกล้เคียง 6 Chunks แต่ในคำถามเปรียบเทียบ 3 โปรเจกต์ โปรเจกต์ที่ 3 จะได้เพียง 1 Chunk</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="34" t="inlineStr">
@@ -3173,7 +3459,7 @@
           <t>Chunks=4, Quota=2 (Compact Balanced)</t>
         </is>
       </c>
-      <c r="C9" s="34" t="inlineStr">
+      <c r="C9" s="35" t="inlineStr">
         <is>
           <t>sweep_chunks_4_quota_2</t>
         </is>
@@ -3232,6 +3518,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T9" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบบริบทขนาดกะทัดรัด (4 Chunks, โควตา 2/โปรเจกต์) เพื่อลดเวลาอ่าน Prompt ของการ์ดจอ</t>
+        </is>
+      </c>
+      <c r="U9" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ ไม่เลือก: เร็วขึ้นเล็กน้อย (13.48s) แต่ได้คะแนน Quality (82.40) และ Phrase Recall (80.0%) ต่ำกว่า 6 Chunks</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="36" t="inlineStr">
@@ -3244,7 +3540,7 @@
           <t>Chunks=2, Quota=1 (Ultra Minimal)</t>
         </is>
       </c>
-      <c r="C10" s="36" t="inlineStr">
+      <c r="C10" s="37" t="inlineStr">
         <is>
           <t>sweep_chunks_2_quota_1</t>
         </is>
@@ -3303,6 +3599,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T10" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบขีดจำกัดล่างสุด (Minimal 2 Chunks, โควตา 1/โปรเจกต์) เพื่อเน้นความเร็วสูงสุด</t>
+        </is>
+      </c>
+      <c r="U10" s="36" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: บริบทน้อยเกินไปสำหรับคำถามเชิงลึกที่รายละเอียดกระจายอยู่หลายหน้า ทำให้ Phrase Recall ลดเหลือ 80.0%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="34" t="inlineStr">
@@ -3315,7 +3621,7 @@
           <t>Chunks=6, Quota=6 (Uncapped / No Quota)</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C11" s="35" t="inlineStr">
         <is>
           <t>sweep_chunks_6_quota_6</t>
         </is>
@@ -3374,6 +3680,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T11" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบส่ง 6 Chunks แต่ปิดการจำกัดโควตาต่อโปรเจกต์ (Uncapped Quota=6) เพื่อพิสูจน์ความสำคัญของ Fair Quota</t>
+        </is>
+      </c>
+      <c r="U11" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือก: เมื่อไม่จำกัดโควตา โปรเจกต์เดียวกินพื้นที่ Chunks จน Input Tokens พุ่งเป็น 2,177 tokens และใช้เวลานานขึ้นเป็น 19.93s</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
@@ -3386,7 +3702,7 @@
           <t>Preset=concise, Temp=0.0, MaxTokens=256</t>
         </is>
       </c>
-      <c r="C12" s="36" t="inlineStr">
+      <c r="C12" s="37" t="inlineStr">
         <is>
           <t>sweep_concise_t00</t>
         </is>
@@ -3445,6 +3761,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T12" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบเปรียบเทียบพารามิเตอร์ฝั่ง LLM</t>
+        </is>
+      </c>
+      <c r="U12" s="36" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="34" t="inlineStr">
@@ -3457,7 +3783,7 @@
           <t>Preset=balanced, Temp=0.0, MaxTokens=384</t>
         </is>
       </c>
-      <c r="C13" s="34" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>sweep_balanced_t00</t>
         </is>
@@ -3516,6 +3842,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T13" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบเปรียบเทียบพารามิเตอร์ฝั่ง LLM</t>
+        </is>
+      </c>
+      <c r="U13" s="34" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="33" t="inlineStr">
@@ -3528,7 +3864,7 @@
           <t>Preset=deep_academic, Temp=0.0, MaxTokens=512</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
         <is>
           <t>sweep_deep_academic_t00</t>
         </is>
@@ -3587,6 +3923,16 @@
           <t>🏆 WINNER</t>
         </is>
       </c>
+      <c r="T14" s="33" t="inlineStr">
+        <is>
+          <t>ทดสอบเปรียบเทียบพารามิเตอร์ฝั่ง LLM</t>
+        </is>
+      </c>
+      <c r="U14" s="33" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="34" t="inlineStr">
@@ -3599,7 +3945,7 @@
           <t>Preset=step_by_step, Temp=0.0, MaxTokens=384</t>
         </is>
       </c>
-      <c r="C15" s="34" t="inlineStr">
+      <c r="C15" s="35" t="inlineStr">
         <is>
           <t>sweep_step_by_step_t00</t>
         </is>
@@ -3658,6 +4004,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T15" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบเปรียบเทียบพารามิเตอร์ฝั่ง LLM</t>
+        </is>
+      </c>
+      <c r="U15" s="34" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="36" t="inlineStr">
@@ -3670,7 +4026,7 @@
           <t>Preset=balanced, Temp=0.2, MaxTokens=384</t>
         </is>
       </c>
-      <c r="C16" s="36" t="inlineStr">
+      <c r="C16" s="37" t="inlineStr">
         <is>
           <t>sweep_balanced_t02</t>
         </is>
@@ -3729,6 +4085,16 @@
           <t>Tested</t>
         </is>
       </c>
+      <c r="T16" s="36" t="inlineStr">
+        <is>
+          <t>ทดสอบเปรียบเทียบพารามิเตอร์ฝั่ง LLM</t>
+        </is>
+      </c>
+      <c r="U16" s="36" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="34" t="inlineStr">
@@ -3741,7 +4107,7 @@
           <t>Preset=balanced, Temp=0.5, MaxTokens=384</t>
         </is>
       </c>
-      <c r="C17" s="34" t="inlineStr">
+      <c r="C17" s="35" t="inlineStr">
         <is>
           <t>sweep_balanced_t05</t>
         </is>
@@ -3798,6 +4164,16 @@
       <c r="S17" s="35" t="inlineStr">
         <is>
           <t>Tested</t>
+        </is>
+      </c>
+      <c r="T17" s="34" t="inlineStr">
+        <is>
+          <t>ทดสอบเปรียบเทียบพารามิเตอร์ฝั่ง LLM</t>
+        </is>
+      </c>
+      <c r="U17" s="34" t="inlineStr">
+        <is>
+          <t>พิจารณาตามคะแนน Composite</t>
         </is>
       </c>
     </row>
@@ -24248,10 +24624,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -24270,7 +24646,8 @@
     <col width="26" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
     <col width="43" customWidth="1" min="19" max="19"/>
-    <col width="52" customWidth="1" min="20" max="20"/>
+    <col width="55" customWidth="1" min="20" max="20"/>
+    <col width="55" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -24386,7 +24763,12 @@
       </c>
       <c r="T4" s="31" t="inlineStr">
         <is>
-          <t>คำแนะนำการใช้งาน (Recommendation)</t>
+          <t>ทำไมถึงนำโมเดลนี้มาทดสอบ (Why Tested / สมมติฐานการทดลอง)</t>
+        </is>
+      </c>
+      <c r="U4" s="31" t="inlineStr">
+        <is>
+          <t>ทำไมถึงเลือก / ไม่เลือกใช้งานจริง (Why Selected / สรุปความคุ้มค่า)</t>
         </is>
       </c>
     </row>
@@ -24460,7 +24842,12 @@
       </c>
       <c r="T5" s="33" t="inlineStr">
         <is>
-          <t>🏆 แนะนำอันดับ 1: รุ่นเล็กของ Meta สำหรับ Laptop GPU 4GB (เด่นภาษาอังกฤษ)</t>
+          <t>นำมาทดสอบเป็นตัวแทนโมเดล 3B มาตรฐานสากลของ Meta ที่ถูกออกแบบมาเพื่อ Laptop GPU ขนาด 4GB โดยเฉพาะ เพื่อดูว่าสกัดรหัสฮาร์ดแวร์และชื่อโครงงานได้แม่นยำเทียบเท่าโมเดล 4B-8B หรือไม่</t>
+        </is>
+      </c>
+      <c r="U5" s="33" t="inlineStr">
+        <is>
+          <t>🏆 เลือกเป็นอันดับ 1 ด้านความคุ้มค่ารวม (Suitability = 87.70): รันบน VRAM 4GB ได้ 100% ตอบไวเฉลี่ย 5.60s (47.6 TPS เร็วกว่า gemma3:4b ถึง 3.4 เท่า) แต่ยังเก็บคำสำคัญ (Phrase Recall 86.7%) และอ้างอิง (Citation 21/30) ได้เทียบเท่ารุ่นใหญ่</t>
         </is>
       </c>
     </row>
@@ -24534,7 +24921,12 @@
       </c>
       <c r="T6" s="33" t="inlineStr">
         <is>
-          <t>🏆 แนะนำอันดับ 2: เน้นความเร็วสูงสุดบน RTX 3050 Ti + แม่นคีย์เวิร์ดไทย/อังกฤษ</t>
+          <t>นำมาทดสอบเป็นตัวแทนโมเดล 3B สายเอเชีย (Alibaba) ขนาดเบา 1.9 GB ที่ไม่ติดโหมดคิดยาว (&lt;think&gt;) เหมือน Qwen 3 เพื่อพิสูจน์ว่าทำสปีดสูงสุดบนการ์ดจอ 4GB โดยยังตอบภาษาไทยได้ดีหรือไม่</t>
+        </is>
+      </c>
+      <c r="U6" s="33" t="inlineStr">
+        <is>
+          <t>🥈 เลือกเป็นอันดับ 2 สายความเร็วสูง (Suitability = 82.48): ปั่น Token เร็วถึง 60.0 TPS กิน VRAM น้อยมาก (1.9 GB) และได้คะแนน Quality 81.20 เหมาะสำหรับโหมดต้องการคำตอบด่วน</t>
         </is>
       </c>
     </row>
@@ -24608,81 +25000,91 @@
       </c>
       <c r="T7" s="34" t="inlineStr">
         <is>
-          <t>Ultra-Lightweight ทดสอบขีดจำกัดความเร็วสูงสุดเมื่อลดขนาดเหลือ 1B</t>
+          <t>นำมาทดสอบเป็นตัวแทน Ultra-Lightweight (1B Parameter, 0.8 GB) เพื่อเป็นขีดจำกัดล่าง (Lower-Bound Control) พิสูจน์ว่าหากลดขนาดโมเดลเหลือ 1B เพื่อเอาความเร็ว &gt;100 TPS คุณภาพคำตอบ RAG จะดรอปลงแค่ไหน</t>
+        </is>
+      </c>
+      <c r="U7" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือกเป็นโมเดลหลัก (ใช้เฉพาะโหมดประหยัดทรัพยากรสุดขีด): แม้เร็วที่สุดถึง 130.7 TPS (6.86s) แต่ขนาด 1B เล็กเกินไปจนเกิดอาการพูดซ้ำ (Repetition) ในข้อ GT-01 และลืมระบุชื่อโครงงาน ทำให้ Phrase Recall ตกเหลือ 66.7%</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="37" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
       </c>
-      <c r="B8" s="36" t="inlineStr">
+      <c r="B8" s="33" t="inlineStr">
         <is>
           <t>gemma3:4b</t>
         </is>
       </c>
-      <c r="C8" s="36" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>Google Gemma 3</t>
         </is>
       </c>
-      <c r="D8" s="37" t="inlineStr">
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>4.3B</t>
         </is>
       </c>
-      <c r="E8" s="37" t="n">
+      <c r="E8" s="32" t="n">
         <v>3.3</v>
       </c>
-      <c r="F8" s="36" t="inlineStr">
+      <c r="F8" s="33" t="inlineStr">
         <is>
           <t>🟢 100% GPU (พอดี VRAM 4GB)</t>
         </is>
       </c>
-      <c r="G8" s="37" t="n">
+      <c r="G8" s="32" t="n">
         <v>21</v>
       </c>
-      <c r="H8" s="37" t="n">
+      <c r="H8" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="I8" s="37" t="n">
+      <c r="I8" s="32" t="n">
         <v>11</v>
       </c>
-      <c r="J8" s="37" t="n">
+      <c r="J8" s="32" t="n">
         <v>18</v>
       </c>
-      <c r="K8" s="37" t="n">
+      <c r="K8" s="32" t="n">
         <v>75</v>
       </c>
-      <c r="L8" s="37" t="n">
+      <c r="L8" s="32" t="n">
         <v>86.68000000000001</v>
       </c>
-      <c r="M8" s="37" t="n">
-        <v>100</v>
-      </c>
-      <c r="N8" s="37" t="n">
-        <v>100</v>
-      </c>
-      <c r="O8" s="37" t="n">
+      <c r="M8" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="N8" s="32" t="n">
+        <v>100</v>
+      </c>
+      <c r="O8" s="32" t="n">
         <v>84.67</v>
       </c>
-      <c r="P8" s="37" t="n">
+      <c r="P8" s="32" t="n">
         <v>90</v>
       </c>
-      <c r="Q8" s="37" t="n">
+      <c r="Q8" s="32" t="n">
         <v>19.23</v>
       </c>
-      <c r="R8" s="37" t="n">
+      <c r="R8" s="32" t="n">
         <v>12.4</v>
       </c>
-      <c r="S8" s="37" t="n">
+      <c r="S8" s="32" t="n">
         <v>78.03</v>
       </c>
-      <c r="T8" s="36" t="inlineStr">
-        <is>
-          <t>Baseline หลัก (สมดุลภาษาไทย-อังกฤษ + โครงสร้าง Markdown)</t>
+      <c r="T8" s="33" t="inlineStr">
+        <is>
+          <t>นำมาทดสอบเป็น Baseline หลักของระบบ (ขนาด 4.3B, 3.3 GB พอดีเพดานการ์ดจอ VRAM 4GB) เนื่องจากตระกูล Gemma 3 โดดเด่นเรื่องการเรียบเรียงภาษาไทยและโครงสร้าง Markdown วิชาการ</t>
+        </is>
+      </c>
+      <c r="U8" s="33" t="inlineStr">
+        <is>
+          <t>🏅 เลือกเป็นแชมป์ด้านคุณภาพเนื้อหาสูงสุด (Quality = 84.67, Phrase Recall = 86.7%): เรียบเรียงคำตอบภาษาไทย ตารางเปรียบเทียบ และอ้างอิง `[Source: ..., Page: ...]` ได้ละเอียดและสละสลวยที่สุด (ใช้เวลาเฉลี่ย 19.23s เพราะเขียนละเอียดถึง ~199 tokens)</t>
         </is>
       </c>
     </row>
@@ -24756,7 +25158,12 @@
       </c>
       <c r="T9" s="34" t="inlineStr">
         <is>
-          <t>ตัวแทนรุ่นกลาง 7B ความเข้าใจลึกซึ้งแต่ใช้เวลาประมวลผลนานขึ้น</t>
+          <t>นำมาทดสอบเป็นตัวแทนรุ่นกลาง 7B Parameter (4.7 GB) เพื่อเป็นกลุ่มเปรียบเทียบ (Upper-Mid Control) ว่าการขยับขนาดเกิน 4GB VRAM เล็กน้อยให้ความแม่นยำเพิ่มขึ้นคุ้มกับความเร็วที่ลดลงหรือไม่</t>
+        </is>
+      </c>
+      <c r="U9" s="34" t="inlineStr">
+        <is>
+          <t>⚠️ ไม่เลือกเป็นค่าเริ่มต้นบนการ์ดจอ 4GB: แม้ได้คะแนน Citation สูงสุด (24/30, Quality 81.80) แต่ขนาด 4.7 GB ล้น VRAM 4GB ต้องสลับใช้ CPU RAM ทำให้ความเร็วลดเหลือ 8.6 TPS (16.97s) ช้ากว่ารุ่น 3B ถึง 5.5 เท่า</t>
         </is>
       </c>
     </row>
@@ -24830,7 +25237,12 @@
       </c>
       <c r="T10" s="36" t="inlineStr">
         <is>
-          <t>รุ่นใหม่เน้นการคิดเชิงเหตุผล (Reasoning) และการสกัดข้อมูลเทคนิค</t>
+          <t>นำมาทดสอบเป็นตัวแทนโมเดลยุคใหม่ที่มีสถาปัตยกรรมคิดเชิงเหตุผล (Reasoning/Thinking) เพื่อดูว่าช่วยวิเคราะห์ตารางเปรียบเทียบโครงงานได้ดีขึ้นหรือไม่</t>
+        </is>
+      </c>
+      <c r="U10" s="36" t="inlineStr">
+        <is>
+          <t>⚠️ ไม่เลือกเป็นค่าเริ่มต้น: โมเดลชอบเขียนแจกแจงขั้นตอนการคิดวิเคราะห์คำถามก่อนเข้าสู่คำตอบจริง (เช่นใน GT-01 และ GT-06) ทำให้เสียโควตา Output Tokens และใช้เวลาตอบนาน (18.20s, Quality 77.73)</t>
         </is>
       </c>
     </row>
@@ -24904,7 +25316,12 @@
       </c>
       <c r="T11" s="34" t="inlineStr">
         <is>
-          <t>ตัวแทนรุ่นใหญ่ 8B มาตรฐานของ Meta</t>
+          <t>นำมาทดสอบเป็นตัวแทนรุ่นใหญ่มาตรฐาน 8B Parameter (4.9 GB) เพื่อเป็นขีดจำกัดบน (Upper-Bound Control) พิสูจน์คอขวดด้านฮาร์ดแวร์เมื่อรันโมเดล 8B บนการ์ดจอ Laptop 4GB VRAM</t>
+        </is>
+      </c>
+      <c r="U11" s="34" t="inlineStr">
+        <is>
+          <t>❌ ไม่เลือกสำหรับ RTX 3050 Ti (4GB VRAM): แม้แม่นยำสูง (Phrase Recall 86.7%, Quality 80.47) แต่ขนาด 4.9 GB ล้น VRAM จนเกิดคอขวด GPU-RAM ความเร็วตกเหลือเพียง 7.3 TPS (เฉลี่ย 20.45s/ข้อ และนานถึง 43.8s ในข้อ GT-01)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(handoff): create RAGcoon_Backend_Frontend_Update_Handoff.xlsx and update existing Excel specs
</commit_message>
<xml_diff>
--- a/backend/data/RAGcoon_Handoff_Specification.xlsx
+++ b/backend/data/RAGcoon_Handoff_Specification.xlsx
@@ -27,6 +27,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_Concrete_Output_Examples" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_LLM_Model_Comparison" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_LLM_PerQuery_Rule_Detail" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21_Backend_Frontend_NextSteps" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -36,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,8 +100,42 @@
       <color rgb="001F4E78"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Tahoma"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <b val="1"/>
+      <color rgb="00334155"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <b val="1"/>
+      <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="000F172A"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Tahoma"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -149,8 +184,26 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9C3"/>
+        <bgColor rgb="00FEF9C3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -186,11 +239,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -266,6 +333,38 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -990,7 +1089,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -1451,7 +1549,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -2406,7 +2503,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -3016,7 +3112,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -4219,7 +4314,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -16185,7 +16279,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -20546,7 +20639,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -23908,7 +24000,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -24353,7 +24444,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -24664,7 +24754,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -26009,7 +26098,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -28189,6 +28277,385 @@
       <c r="P39" s="34" t="inlineStr">
         <is>
           <t>## Comparison Overview | Dimension | The LoRaWAN | Beacon Signal Location Device | |---|---|---| | ฮาร์ดแวร์ | TTGO และ ESP32 | ไม่ระบุ |  ## Key Differences - ฮาร์ดแวร์ที่ใช้ของ The LoRaWAN คือ TTGO และ ESP32 ในขณะที่ไม่ระบุฮาร์ดแวร์ที่ใช้</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>🚀 แผนส่งมอบงานให้ทีม Backend &amp; Frontend อัปเดตต่อ (Backend &amp; Frontend Update Action Plan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>สรุปรายการที่ทีม Backend (FastAPI) และทีม Frontend (UI) ต้องนำไปอัปเดตต่อหลังจากจบการจูนพารามิเตอร์และทดสอบ LLM ทั้ง 7 รุ่น</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="40" t="inlineStr">
+        <is>
+          <t>รหัสงาน (Task ID)</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="inlineStr">
+        <is>
+          <t>ความสำคัญ (Priority)</t>
+        </is>
+      </c>
+      <c r="C4" s="40" t="inlineStr">
+        <is>
+          <t>ทีมรับผิดชอบ (Owner)</t>
+        </is>
+      </c>
+      <c r="D4" s="40" t="inlineStr">
+        <is>
+          <t>หัวข้อสิ่งที่ต้องทำเพิ่ม (Action Item)</t>
+        </is>
+      </c>
+      <c r="E4" s="40" t="inlineStr">
+        <is>
+          <t>ไฟล์ที่ต้องแก้ไข / สร้างเพิ่ม (Target Files)</t>
+        </is>
+      </c>
+      <c r="F4" s="40" t="inlineStr">
+        <is>
+          <t>สาเหตุและสิ่งที่ฝั่ง RAG เตรียมไว้ให้แล้ว (Why Needed &amp; What RAG Already Built)</t>
+        </is>
+      </c>
+      <c r="G4" s="40" t="inlineStr">
+        <is>
+          <t>รายละเอียดการอัปเดตที่ต้องทำ (Exact Implementation Steps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>ACT-01</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>P0 (ด่วนที่สุด)</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Backend (FastAPI)</t>
+        </is>
+      </c>
+      <c r="D5" s="42" t="inlineStr">
+        <is>
+          <t>อัปเดต ChatRequest &amp; rag_services.py ให้ส่งต่อ llm_model, llm_provider และ config</t>
+        </is>
+      </c>
+      <c r="E5" s="43" t="inlineStr">
+        <is>
+          <t>backend/app/schemas/chat.py
+backend/app/services/rag_services.py
+backend/app/api/v1/chat.py</t>
+        </is>
+      </c>
+      <c r="F5" s="42" t="inlineStr">
+        <is>
+          <t>ปัจจุบัน answer_question() และ stream_answer_question() ในฝั่ง RAG รองรับการเปลี่ยนโมเดล (7 รุ่น) และโปรไฟล์พารามิเตอร์แล้ว แต่ rag_services.py บรรทัด 136 และ 220 ยังเรียกแบบไม่ส่งพารามิเตอร์ ทำให้ผู้ใช้เลือกโมเดลหรือโปรไฟล์รายคำถามไม่ได้</t>
+        </is>
+      </c>
+      <c r="G5" s="42" t="inlineStr">
+        <is>
+          <t>เพิ่มฟิลด์ llm_provider, llm_model, profile_name ใน ChatRequest และส่งเข้าไปใน answer_question() / stream_answer_question()</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="88" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>ACT-02</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>P0 (ด่วนที่สุด)</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Backend &amp; DevOps</t>
+        </is>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>อัปเดตค่า Default พารามิเตอร์และโมเดลตามผลการทดลองที่ชนะเลิศ (Optimal Tuned Lock)</t>
+        </is>
+      </c>
+      <c r="E6" s="43" t="inlineStr">
+        <is>
+          <t>backend/app/rag/retrieval/rag_config.py
+backend/.env
+docker-compose.yml</t>
+        </is>
+      </c>
+      <c r="F6" s="42" t="inlineStr">
+        <is>
+          <t>ผลการทดลองพิสูจน์แล้วว่า top_k=15, rerank_top_n=10, max_context_chunks=6, max_chunks_per_project=2, temp=0.0 ให้ Hit Rate 100%, MRR 0.9231 และ Quality 84.67 โดยเร็วขึ้นกว่าเดิมมาก ส่วนโมเดลบน RTX 3050 Ti แนะนำ llama3.2:3b (ไว 5.6s) และ gemma3:4b (ภาษาไทยละเอียดสุด)</t>
+        </is>
+      </c>
+      <c r="G6" s="42" t="inlineStr">
+        <is>
+          <t>ตั้งค่าเริ่มต้นใน .env หรือให้ระบบใช้ Active Profile จาก rag_config.py (ตั้งค่าเริ่มต้นแล้ว) และรัน docker-compose up เพื่อให้ Container ollama ดึงโมเดลทั้ง 6-7 รุ่นอัตโนมัติ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>ACT-03</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>P0 (ด่วนที่สุด)</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Frontend (UI)</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>สร้าง Dropdown สลับโมเดล LLM ทั้ง 7 รุ่น บนหน้า Chat พร้อมป้ายแนะนำความเร็ว/VRAM</t>
+        </is>
+      </c>
+      <c r="E7" s="43" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Chat/... (Chat Header / Model Selector)</t>
+        </is>
+      </c>
+      <c r="F7" s="42" t="inlineStr">
+        <is>
+          <t>ฝั่ง RAG ได้ติดตั้งและทดสอบโมเดล 7 รุ่นใน AVAILABLE_LLM_PROFILES เรียบร้อยแล้ว ผู้ใช้ควรเลือกสลับโหมดได้ตามงาน เช่น โหมดตอบไว (llama3.2:3b / qwen2.5:3b) หรือโหมดวิชาการละเอียด (gemma3:4b)</t>
+        </is>
+      </c>
+      <c r="G7" s="42" t="inlineStr">
+        <is>
+          <t>เรียก GET /api/v1/chat/llm-profiles เพื่อแสดงรายการโมเดล และเรียก POST /api/v1/chat/set-active-llm หรือส่ง llm_model ไปกับ POST /api/v1/chat/query-stream</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="44" t="inlineStr">
+        <is>
+          <t>ACT-04</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="inlineStr">
+        <is>
+          <t>P1 (สำคัญมาก)</t>
+        </is>
+      </c>
+      <c r="C8" s="44" t="inlineStr">
+        <is>
+          <t>Backend (FastAPI)</t>
+        </is>
+      </c>
+      <c r="D8" s="45" t="inlineStr">
+        <is>
+          <t>เปิดใช้งาน API Endpoints สำหรับปรับจูนพารามิเตอร์อิสระและเซฟโปรไฟล์ใหม่ (RAG Config API)</t>
+        </is>
+      </c>
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>backend/app/api/v1/ai_config.py (สร้างใหม่)
+backend/app/api/v1/router.py</t>
+        </is>
+      </c>
+      <c r="F8" s="45" t="inlineStr">
+        <is>
+          <t>ฝั่ง RAG สร้างฟังก์ชัน list_all_configs(), save_custom_config(), set_active_rag_config_by_name(), delete_custom_config() และ compare_two_configs() ไว้เสร็จสมบูรณ์แล้ว แต่ยังไม่มี Route ใน api/v1/router.py ให้ Frontend เรียกใช้</t>
+        </is>
+      </c>
+      <c r="G8" s="45" t="inlineStr">
+        <is>
+          <t>สร้าง Router `/api/v1/rag-config` ผูกเข้ากับฟังก์ชันใน `app.rag.retrieval.rag_config` และ `app.rag.evaluation.config_benchmark` (มีโค้ดตัวอย่างให้ใน Sheet 03 และ Sheet 04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>ACT-05</t>
+        </is>
+      </c>
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>P1 (สำคัญมาก)</t>
+        </is>
+      </c>
+      <c r="C9" s="44" t="inlineStr">
+        <is>
+          <t>Frontend (UI)</t>
+        </is>
+      </c>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>สร้างหน้าจอ Admin RAG Parameter Studio (Sliders + Toggles เปิด/ปิดโมดูล + ปุ่ม Save as New Profile)</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>frontend/src/pages/admin/... (AI Config / Parameter Studio)</t>
+        </is>
+      </c>
+      <c r="F9" s="45" t="inlineStr">
+        <is>
+          <t>เพื่อให้ผู้ดูแลระบบปรับค่า top_k [5..100], rerank_top_n [1..30], max_context_chunks [2..15], max_chunks_per_project [1..5], เปิด/ปิด Hybrid BM25, Reranker, Boilerplate Filter, Fast-Path และเซฟเป็นโปรไฟล์ทดสอบชื่อใหม่ผ่านหน้าเว็บได้ทันที</t>
+        </is>
+      </c>
+      <c r="G9" s="45" t="inlineStr">
+        <is>
+          <t>สร้าง UI Sliders + Switch Toggles เชื่อมกับ POST /api/v1/rag-config/profiles และปุ่มเปรียบเทียบโปรไฟล์เก่า vs ใหม่ (POST /api/v1/rag-config/compare)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="44" t="inlineStr">
+        <is>
+          <t>ACT-06</t>
+        </is>
+      </c>
+      <c r="B10" s="44" t="inlineStr">
+        <is>
+          <t>P1 (สำคัญมาก)</t>
+        </is>
+      </c>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>Backend &amp; Frontend</t>
+        </is>
+      </c>
+      <c r="D10" s="45" t="inlineStr">
+        <is>
+          <t>ส่งข้อมูล Performance Metrics (ความเร็ว TPS, Input/Output Tokens, Token Breakdown) ไปแสดงใต้คำตอบ</t>
+        </is>
+      </c>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>backend/app/schemas/chat.py
+backend/app/services/rag_services.py
+frontend/src/components/Chat/MessageItem</t>
+        </is>
+      </c>
+      <c r="F10" s="45" t="inlineStr">
+        <is>
+          <t>ฝั่ง RAG คำนวณ gen_speed_tps, input_tokens, output_tokens และ token_breakdown ส่งออกมาใน dict `performance` แล้ว แต่ rag_services.py ตัดทิ้งก่อนส่งให้ Frontend</t>
+        </is>
+      </c>
+      <c r="G10" s="45" t="inlineStr">
+        <is>
+          <t>เพิ่มฟิลด์ `performance` และ `model` ใน ChatResponse และใน SSE `metadata` event เพื่อให้ Frontend แสดงป้ายกำกับ เช่น `⚡ 47.6 TPS | ⏱️ 5.6s | 🪙 1,519 in / 93 out tokens | 🤖 llama3.2:3b`</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1">
+      <c r="A11" s="44" t="inlineStr">
+        <is>
+          <t>ACT-07</t>
+        </is>
+      </c>
+      <c r="B11" s="44" t="inlineStr">
+        <is>
+          <t>P1 (สำคัญมาก)</t>
+        </is>
+      </c>
+      <c r="C11" s="44" t="inlineStr">
+        <is>
+          <t>Frontend (UI)</t>
+        </is>
+      </c>
+      <c r="D11" s="45" t="inlineStr">
+        <is>
+          <t>อัปเกรดการ์ดเอกสารอ้างอิง (Citation Card) ให้แสดงเลขหน้ารวม (pages_formatted) และข้อมูลโครงงานครบถ้วน</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>frontend/src/components/Chat/CitationCard</t>
+        </is>
+      </c>
+      <c r="F11" s="45" t="inlineStr">
+        <is>
+          <t>ฝั่ง RAG ได้ยุบรวม Chunks จากไฟล์เดียวกันและสร้างฟิลด์ `pages_formatted` (เช่น '17, 18, 22'), `author`, `advisor`, `year`, `program` ส่งมาใน `citations` เรียบร้อยแล้ว</t>
+        </is>
+      </c>
+      <c r="G11" s="45" t="inlineStr">
+        <is>
+          <t>แสดงเลขหน้าทั้งหมดจาก `citation.pages_formatted` แสดงชื่อผู้จัดทำ/อาจารย์ที่ปรึกษา และทำลิงก์คลิกเปิด PDF ไปยังเลขหน้าเริ่มต้น (`/api/v1/documents/{document_id}/file#page={page}`)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1">
+      <c r="A12" s="47" t="inlineStr">
+        <is>
+          <t>ACT-08</t>
+        </is>
+      </c>
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t>P2 (ต่อยอด)</t>
+        </is>
+      </c>
+      <c r="C12" s="47" t="inlineStr">
+        <is>
+          <t>Backend &amp; Frontend</t>
+        </is>
+      </c>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>เพิ่มหน้า Dashboard แสดงผลการทดลองจูนพารามิเตอร์และตารางจัดอันดับ LLM 7 รุ่น</t>
+        </is>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>backend/app/api/v1/dashboard.py
+frontend/src/pages/admin/dashboard</t>
+        </is>
+      </c>
+      <c r="F12" s="48" t="inlineStr">
+        <is>
+          <t>มีไฟล์ผลลัพธ์มาตรฐาน `data/parameter_sweep_results.json` และ `best_rag_config.json` ที่เก็บผลลัพธ์ครบทั้ง Stage 1, Stage 2 และ Stage 3 (7 โมเดล LLM) พร้อมกฎการให้คะแนน Rule 1-7</t>
+        </is>
+      </c>
+      <c r="G12" s="48" t="inlineStr">
+        <is>
+          <t>เพิ่ม Endpoint `GET /api/v1/dashboard/rag-benchmark` อ่านไฟล์ `parameter_sweep_results.json` ส่งให้ Frontend วาดกราฟเปรียบเทียบความแม่นยำและความเร็วของแต่ละพารามิเตอร์/โมเดล</t>
         </is>
       </c>
     </row>

</xml_diff>